<commit_message>
feat: add column sorting and PO number search functionality
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="511">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="529">
   <x:si>
     <x:t>Document No</x:t>
   </x:si>
@@ -396,7 +396,7 @@
     <x:t>SAPO26010110</x:t>
   </x:si>
   <x:si>
-    <x:t>HOIST Module</x:t>
+    <x:t>HOIST</x:t>
   </x:si>
   <x:si>
     <x:t>F1 20MM wide Elatech Italy Open-End Black PU/Polyurethane Steel Cord Flat Belt</x:t>
@@ -1026,9 +1026,6 @@
   </x:si>
   <x:si>
     <x:t>OMRP513-F3005-00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HOIST</x:t>
   </x:si>
   <x:si>
     <x:t>OMRP513-F2001-00</x:t>
@@ -1245,6 +1242,9 @@
     <x:t>height sensor</x:t>
   </x:si>
   <x:si>
+    <x:t>Banner</x:t>
+  </x:si>
+  <x:si>
     <x:t>A0-139452_EP01</x:t>
   </x:si>
   <x:si>
@@ -1263,10 +1263,20 @@
     <x:t>C-SX2RL24-L_b</x:t>
   </x:si>
   <x:si>
+    <x:t>RFQ4134551</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RFQ Reject</x:t>
+  </x:si>
+  <x:si>
+    <x:t>clamp plate</x:t>
+  </x:si>
+  <x:si>
     <x:t>RFQ4129252</x:t>
   </x:si>
   <x:si>
-    <x:t>clamp plate</x:t>
+    <x:t xml:space="preserve">https://internal.sophicauto.net/BOM/downloadFile/45809
+</x:t>
   </x:si>
   <x:si>
     <x:t>motor</x:t>
@@ -1276,6 +1286,22 @@
   </x:si>
   <x:si>
     <x:t>PVD-PX110-100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RFQ4133271</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PR5327031</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fulitech Technology Co. Limited</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">https://internal.sophicauto.net/BOM/downloadFile/46660
+</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAPO26030523</x:t>
   </x:si>
   <x:si>
     <x:t>Pivot Pin</x:t>
@@ -1321,9 +1347,6 @@
     <x:t>PR5319341</x:t>
   </x:si>
   <x:si>
-    <x:t>Fulitech Technology Co. Limited</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://internal.sophicauto.net/BOM/downloadFile/45744
 </x:t>
   </x:si>
@@ -1339,9 +1362,6 @@
 </x:t>
   </x:si>
   <x:si>
-    <x:t>RFQ Reject</x:t>
-  </x:si>
-  <x:si>
     <x:t>Linear Guide Bearing</x:t>
   </x:si>
   <x:si>
@@ -1483,9 +1503,6 @@
     <x:t>SAPO26030296</x:t>
   </x:si>
   <x:si>
-    <x:t>RFQ Approved</x:t>
-  </x:si>
-  <x:si>
     <x:t>misumi [YHD]</x:t>
   </x:si>
   <x:si>
@@ -1493,12 +1510,18 @@
   </x:si>
   <x:si>
     <x:t>RFQ4130402</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PR5327071</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://internal.sophicauto.net/BOM/downloadFile/46459
 </x:t>
   </x:si>
   <x:si>
+    <x:t>SAPO26030524</x:t>
+  </x:si>
+  <x:si>
     <x:t>ball plungers</x:t>
   </x:si>
   <x:si>
@@ -1560,12 +1583,18 @@
   </x:si>
   <x:si>
     <x:t>RFQ4130871</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PR5328791</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://internal.sophicauto.net/BOM/downloadFile/45815
 </x:t>
   </x:si>
   <x:si>
+    <x:t>SAPO26030607</x:t>
+  </x:si>
+  <x:si>
     <x:t>OMR-STR-F1124A</x:t>
   </x:si>
   <x:si>
@@ -1628,6 +1657,33 @@
   </x:si>
   <x:si>
     <x:t>SHIPPING</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Track</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OMR-2701A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RFQ4133302</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OMR-2702A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OMR-2705A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OMR-2706A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OMR-2703A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RFQ4133662</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OMR-2704A</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2016,7 +2072,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:AC198"/>
+  <x:dimension ref="A1:AC204"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="30" max="16384" width="9.140625" style="1" customWidth="1"/>
@@ -3505,7 +3561,7 @@
     </x:row>
     <x:row r="27" spans="1:29">
       <x:c r="A27" s="4">
-        <x:v>46029.6167459838</x:v>
+        <x:v>46113.7096591435</x:v>
       </x:c>
       <x:c r="B27" s="1" t="n">
         <x:v>32341</x:v>
@@ -8598,10 +8654,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D103" s="1" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="E103" s="1" t="s">
         <x:v>328</x:v>
-      </x:c>
-      <x:c r="E103" s="1" t="s">
-        <x:v>329</x:v>
       </x:c>
       <x:c r="F103" s="1" t="s">
         <x:v>51</x:v>
@@ -8622,13 +8678,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M103" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N103" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O103" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P103" s="1" t="n">
         <x:v>70</x:v>
@@ -8640,13 +8696,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S103" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T103" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U103" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T103" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U103" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V103" s="1" t="n">
         <x:v>4</x:v>
@@ -8666,10 +8722,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D104" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E104" s="1" t="s">
-        <x:v>334</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="F104" s="1" t="s">
         <x:v>51</x:v>
@@ -8690,13 +8746,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M104" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N104" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O104" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P104" s="1" t="n">
         <x:v>35</x:v>
@@ -8708,13 +8764,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S104" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T104" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U104" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T104" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U104" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V104" s="1" t="n">
         <x:v>1</x:v>
@@ -8734,10 +8790,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D105" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E105" s="1" t="s">
-        <x:v>335</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="F105" s="1" t="s">
         <x:v>51</x:v>
@@ -8758,13 +8814,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M105" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N105" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O105" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P105" s="1" t="n">
         <x:v>85</x:v>
@@ -8776,13 +8832,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S105" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T105" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U105" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T105" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U105" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V105" s="1" t="n">
         <x:v>2</x:v>
@@ -8802,10 +8858,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D106" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E106" s="1" t="s">
-        <x:v>336</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="F106" s="1" t="s">
         <x:v>51</x:v>
@@ -8826,13 +8882,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M106" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N106" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O106" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P106" s="1" t="n">
         <x:v>275</x:v>
@@ -8844,13 +8900,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S106" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T106" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U106" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T106" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U106" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V106" s="1" t="n">
         <x:v>1</x:v>
@@ -8870,10 +8926,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D107" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E107" s="1" t="s">
-        <x:v>337</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="F107" s="1" t="s">
         <x:v>51</x:v>
@@ -8894,13 +8950,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M107" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N107" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O107" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P107" s="1" t="n">
         <x:v>50</x:v>
@@ -8912,13 +8968,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S107" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T107" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U107" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T107" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U107" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V107" s="1" t="n">
         <x:v>12</x:v>
@@ -8938,10 +8994,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D108" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E108" s="1" t="s">
-        <x:v>338</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="F108" s="1" t="s">
         <x:v>51</x:v>
@@ -8962,13 +9018,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M108" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N108" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O108" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P108" s="1" t="n">
         <x:v>25</x:v>
@@ -8980,13 +9036,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S108" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T108" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U108" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T108" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U108" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V108" s="1" t="n">
         <x:v>6</x:v>
@@ -9006,10 +9062,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D109" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E109" s="1" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="F109" s="1" t="s">
         <x:v>51</x:v>
@@ -9030,13 +9086,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M109" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N109" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O109" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P109" s="1" t="n">
         <x:v>100</x:v>
@@ -9048,13 +9104,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S109" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T109" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U109" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T109" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U109" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V109" s="1" t="n">
         <x:v>2</x:v>
@@ -9074,10 +9130,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D110" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E110" s="1" t="s">
-        <x:v>340</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="F110" s="1" t="s">
         <x:v>51</x:v>
@@ -9098,13 +9154,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M110" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N110" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O110" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P110" s="1" t="n">
         <x:v>20</x:v>
@@ -9116,13 +9172,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S110" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T110" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U110" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T110" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U110" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V110" s="1" t="n">
         <x:v>12</x:v>
@@ -9142,10 +9198,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D111" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E111" s="1" t="s">
-        <x:v>341</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="F111" s="1" t="s">
         <x:v>51</x:v>
@@ -9166,13 +9222,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M111" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N111" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O111" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P111" s="1" t="n">
         <x:v>155</x:v>
@@ -9184,13 +9240,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S111" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T111" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U111" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T111" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U111" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V111" s="1" t="n">
         <x:v>1</x:v>
@@ -9210,10 +9266,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D112" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E112" s="1" t="s">
-        <x:v>342</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="F112" s="1" t="s">
         <x:v>51</x:v>
@@ -9234,13 +9290,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M112" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N112" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O112" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P112" s="1" t="n">
         <x:v>135</x:v>
@@ -9252,13 +9308,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S112" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T112" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U112" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T112" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U112" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V112" s="1" t="n">
         <x:v>4</x:v>
@@ -9278,10 +9334,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D113" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E113" s="1" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="F113" s="1" t="s">
         <x:v>51</x:v>
@@ -9302,13 +9358,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M113" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N113" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O113" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P113" s="1" t="n">
         <x:v>25</x:v>
@@ -9320,13 +9376,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S113" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T113" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U113" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T113" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U113" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V113" s="1" t="n">
         <x:v>2</x:v>
@@ -9346,10 +9402,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D114" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E114" s="1" t="s">
-        <x:v>344</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="F114" s="1" t="s">
         <x:v>51</x:v>
@@ -9370,13 +9426,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M114" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N114" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O114" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P114" s="1" t="n">
         <x:v>20</x:v>
@@ -9388,13 +9444,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S114" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T114" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U114" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T114" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U114" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V114" s="1" t="n">
         <x:v>2</x:v>
@@ -9414,10 +9470,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D115" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E115" s="1" t="s">
-        <x:v>345</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="F115" s="1" t="s">
         <x:v>51</x:v>
@@ -9438,13 +9494,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M115" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N115" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O115" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P115" s="1" t="n">
         <x:v>80</x:v>
@@ -9456,13 +9512,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S115" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T115" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U115" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T115" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U115" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V115" s="1" t="n">
         <x:v>2</x:v>
@@ -9482,10 +9538,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D116" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E116" s="1" t="s">
-        <x:v>346</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="F116" s="1" t="s">
         <x:v>51</x:v>
@@ -9506,13 +9562,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M116" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N116" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O116" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P116" s="1" t="n">
         <x:v>15</x:v>
@@ -9524,13 +9580,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S116" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T116" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U116" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T116" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U116" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V116" s="1" t="n">
         <x:v>8</x:v>
@@ -9550,10 +9606,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D117" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E117" s="1" t="s">
-        <x:v>347</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="F117" s="1" t="s">
         <x:v>51</x:v>
@@ -9574,13 +9630,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M117" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N117" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O117" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P117" s="1" t="n">
         <x:v>18</x:v>
@@ -9592,13 +9648,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S117" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T117" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U117" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T117" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U117" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V117" s="1" t="n">
         <x:v>4</x:v>
@@ -9618,10 +9674,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D118" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E118" s="1" t="s">
-        <x:v>348</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="F118" s="1" t="s">
         <x:v>51</x:v>
@@ -9642,13 +9698,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M118" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N118" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O118" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P118" s="1" t="n">
         <x:v>20</x:v>
@@ -9660,13 +9716,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S118" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T118" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U118" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T118" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U118" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V118" s="1" t="n">
         <x:v>2</x:v>
@@ -9686,10 +9742,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D119" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E119" s="1" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="F119" s="1" t="s">
         <x:v>51</x:v>
@@ -9710,13 +9766,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M119" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N119" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O119" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P119" s="1" t="n">
         <x:v>20</x:v>
@@ -9728,13 +9784,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S119" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T119" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U119" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T119" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U119" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V119" s="1" t="n">
         <x:v>2</x:v>
@@ -9754,10 +9810,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D120" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E120" s="1" t="s">
-        <x:v>350</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="F120" s="1" t="s">
         <x:v>51</x:v>
@@ -9778,13 +9834,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M120" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N120" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O120" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P120" s="1" t="n">
         <x:v>60</x:v>
@@ -9796,13 +9852,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S120" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T120" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U120" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T120" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U120" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V120" s="1" t="n">
         <x:v>4</x:v>
@@ -9822,10 +9878,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D121" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E121" s="1" t="s">
-        <x:v>351</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="F121" s="1" t="s">
         <x:v>51</x:v>
@@ -9846,13 +9902,13 @@
         <x:v>46093.4548872338</x:v>
       </x:c>
       <x:c r="M121" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="N121" s="4">
         <x:v>46093.4565539005</x:v>
       </x:c>
       <x:c r="O121" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P121" s="1" t="n">
         <x:v>45</x:v>
@@ -9864,13 +9920,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S121" s="1" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="T121" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U121" s="1" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="T121" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U121" s="1" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="V121" s="1" t="n">
         <x:v>4</x:v>
@@ -9890,10 +9946,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D122" s="1" t="s">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="E122" s="1" t="s">
         <x:v>352</x:v>
-      </x:c>
-      <x:c r="E122" s="1" t="s">
-        <x:v>353</x:v>
       </x:c>
       <x:c r="F122" s="1" t="s">
         <x:v>51</x:v>
@@ -9914,13 +9970,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M122" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N122" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O122" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P122" s="1" t="n">
         <x:v>25</x:v>
@@ -9932,13 +9988,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S122" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T122" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U122" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T122" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U122" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V122" s="1" t="n">
         <x:v>6</x:v>
@@ -9958,10 +10014,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D123" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E123" s="1" t="s">
-        <x:v>358</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="F123" s="1" t="s">
         <x:v>51</x:v>
@@ -9982,13 +10038,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M123" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N123" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O123" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P123" s="1" t="n">
         <x:v>70</x:v>
@@ -10000,13 +10056,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S123" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T123" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U123" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T123" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U123" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V123" s="1" t="n">
         <x:v>2</x:v>
@@ -10026,10 +10082,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D124" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E124" s="1" t="s">
-        <x:v>359</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="F124" s="1" t="s">
         <x:v>51</x:v>
@@ -10050,13 +10106,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M124" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N124" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O124" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P124" s="1" t="n">
         <x:v>40</x:v>
@@ -10068,13 +10124,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S124" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T124" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U124" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T124" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U124" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V124" s="1" t="n">
         <x:v>4</x:v>
@@ -10094,10 +10150,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D125" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E125" s="1" t="s">
-        <x:v>360</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="F125" s="1" t="s">
         <x:v>51</x:v>
@@ -10118,13 +10174,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M125" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N125" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O125" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P125" s="1" t="n">
         <x:v>85</x:v>
@@ -10136,13 +10192,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S125" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T125" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U125" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T125" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U125" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V125" s="1" t="n">
         <x:v>2</x:v>
@@ -10162,10 +10218,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D126" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E126" s="1" t="s">
-        <x:v>361</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="F126" s="1" t="s">
         <x:v>51</x:v>
@@ -10186,13 +10242,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M126" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N126" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O126" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P126" s="1" t="n">
         <x:v>120</x:v>
@@ -10204,13 +10260,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S126" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T126" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U126" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T126" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U126" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V126" s="1" t="n">
         <x:v>4</x:v>
@@ -10230,10 +10286,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D127" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E127" s="1" t="s">
-        <x:v>362</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="F127" s="1" t="s">
         <x:v>51</x:v>
@@ -10254,13 +10310,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M127" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N127" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O127" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P127" s="1" t="n">
         <x:v>40</x:v>
@@ -10272,13 +10328,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S127" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T127" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U127" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T127" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U127" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V127" s="1" t="n">
         <x:v>4</x:v>
@@ -10298,10 +10354,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D128" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E128" s="1" t="s">
-        <x:v>363</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="F128" s="1" t="s">
         <x:v>51</x:v>
@@ -10322,13 +10378,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M128" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N128" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O128" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P128" s="1" t="n">
         <x:v>100</x:v>
@@ -10340,13 +10396,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S128" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T128" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U128" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T128" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U128" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V128" s="1" t="n">
         <x:v>4</x:v>
@@ -10366,10 +10422,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D129" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E129" s="1" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="F129" s="1" t="s">
         <x:v>51</x:v>
@@ -10390,13 +10446,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M129" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N129" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O129" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P129" s="1" t="n">
         <x:v>80</x:v>
@@ -10408,13 +10464,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S129" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T129" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U129" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T129" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U129" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V129" s="1" t="n">
         <x:v>4</x:v>
@@ -10434,10 +10490,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D130" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E130" s="1" t="s">
-        <x:v>365</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="F130" s="1" t="s">
         <x:v>51</x:v>
@@ -10458,13 +10514,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M130" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N130" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O130" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P130" s="1" t="n">
         <x:v>25</x:v>
@@ -10476,13 +10532,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S130" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T130" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U130" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T130" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U130" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V130" s="1" t="n">
         <x:v>2</x:v>
@@ -10502,10 +10558,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D131" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E131" s="1" t="s">
-        <x:v>366</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="F131" s="1" t="s">
         <x:v>51</x:v>
@@ -10526,13 +10582,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M131" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N131" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O131" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P131" s="1" t="n">
         <x:v>50</x:v>
@@ -10544,13 +10600,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S131" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T131" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U131" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T131" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U131" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V131" s="1" t="n">
         <x:v>2</x:v>
@@ -10570,10 +10626,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D132" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E132" s="1" t="s">
-        <x:v>367</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="F132" s="1" t="s">
         <x:v>51</x:v>
@@ -10594,13 +10650,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M132" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N132" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O132" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P132" s="1" t="n">
         <x:v>40</x:v>
@@ -10612,13 +10668,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S132" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T132" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U132" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T132" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U132" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V132" s="1" t="n">
         <x:v>2</x:v>
@@ -10638,10 +10694,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D133" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E133" s="1" t="s">
-        <x:v>368</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="F133" s="1" t="s">
         <x:v>51</x:v>
@@ -10662,13 +10718,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M133" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N133" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O133" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P133" s="1" t="n">
         <x:v>65</x:v>
@@ -10680,13 +10736,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S133" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T133" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U133" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T133" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U133" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V133" s="1" t="n">
         <x:v>1</x:v>
@@ -10706,10 +10762,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D134" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E134" s="1" t="s">
-        <x:v>369</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="F134" s="1" t="s">
         <x:v>51</x:v>
@@ -10730,13 +10786,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M134" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N134" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O134" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P134" s="1" t="n">
         <x:v>45</x:v>
@@ -10748,13 +10804,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S134" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T134" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U134" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T134" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U134" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V134" s="1" t="n">
         <x:v>1</x:v>
@@ -10774,10 +10830,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D135" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E135" s="1" t="s">
-        <x:v>370</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="F135" s="1" t="s">
         <x:v>51</x:v>
@@ -10798,13 +10854,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M135" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N135" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O135" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P135" s="1" t="n">
         <x:v>17</x:v>
@@ -10816,13 +10872,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S135" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T135" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U135" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T135" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U135" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V135" s="1" t="n">
         <x:v>1</x:v>
@@ -10842,10 +10898,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D136" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E136" s="1" t="s">
-        <x:v>371</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="F136" s="1" t="s">
         <x:v>51</x:v>
@@ -10866,13 +10922,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M136" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N136" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O136" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P136" s="1" t="n">
         <x:v>30</x:v>
@@ -10884,13 +10940,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S136" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T136" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U136" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T136" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U136" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V136" s="1" t="n">
         <x:v>2</x:v>
@@ -10910,10 +10966,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D137" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E137" s="1" t="s">
-        <x:v>372</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="F137" s="1" t="s">
         <x:v>51</x:v>
@@ -10934,13 +10990,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M137" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N137" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O137" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P137" s="1" t="n">
         <x:v>40</x:v>
@@ -10952,13 +11008,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S137" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T137" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U137" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T137" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U137" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V137" s="1" t="n">
         <x:v>1</x:v>
@@ -10978,10 +11034,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D138" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E138" s="1" t="s">
-        <x:v>373</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="F138" s="1" t="s">
         <x:v>51</x:v>
@@ -11002,13 +11058,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M138" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N138" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O138" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P138" s="1" t="n">
         <x:v>320</x:v>
@@ -11020,13 +11076,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S138" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T138" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U138" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T138" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U138" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V138" s="1" t="n">
         <x:v>1</x:v>
@@ -11046,10 +11102,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D139" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E139" s="1" t="s">
-        <x:v>374</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="F139" s="1" t="s">
         <x:v>51</x:v>
@@ -11070,13 +11126,13 @@
         <x:v>46092.8395457523</x:v>
       </x:c>
       <x:c r="M139" s="1" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="N139" s="4">
         <x:v>46092.8408331366</x:v>
       </x:c>
       <x:c r="O139" s="1" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="P139" s="1" t="n">
         <x:v>18</x:v>
@@ -11088,13 +11144,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S139" s="1" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="T139" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U139" s="1" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="T139" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U139" s="1" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="V139" s="1" t="n">
         <x:v>1</x:v>
@@ -11111,13 +11167,13 @@
         <x:v>35841</x:v>
       </x:c>
       <x:c r="C140" s="1" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="D140" s="1" t="s">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="E140" s="1" t="s">
         <x:v>375</x:v>
-      </x:c>
-      <x:c r="D140" s="1" t="s">
-        <x:v>352</x:v>
-      </x:c>
-      <x:c r="E140" s="1" t="s">
-        <x:v>376</x:v>
       </x:c>
       <x:c r="F140" s="1" t="s">
         <x:v>158</x:v>
@@ -11138,13 +11194,13 @@
         <x:v>46076.6465126505</x:v>
       </x:c>
       <x:c r="M140" s="1" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="R140" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
       <x:c r="S140" s="1" t="s">
-        <x:v>378</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="T140" s="1" t="n">
         <x:v>1</x:v>
@@ -11158,13 +11214,13 @@
         <x:v>35842</x:v>
       </x:c>
       <x:c r="C141" s="1" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="D141" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E141" s="1" t="s">
-        <x:v>379</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="F141" s="1" t="s">
         <x:v>158</x:v>
@@ -11185,13 +11241,13 @@
         <x:v>46076.6465126505</x:v>
       </x:c>
       <x:c r="M141" s="1" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="R141" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
       <x:c r="S141" s="1" t="s">
-        <x:v>378</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="T141" s="1" t="n">
         <x:v>1</x:v>
@@ -11205,13 +11261,13 @@
         <x:v>35843</x:v>
       </x:c>
       <x:c r="C142" s="1" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="D142" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E142" s="1" t="s">
-        <x:v>380</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="F142" s="1" t="s">
         <x:v>158</x:v>
@@ -11232,13 +11288,13 @@
         <x:v>46076.6465126505</x:v>
       </x:c>
       <x:c r="M142" s="1" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="R142" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
       <x:c r="S142" s="1" t="s">
-        <x:v>378</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="T142" s="1" t="n">
         <x:v>1</x:v>
@@ -11252,13 +11308,13 @@
         <x:v>35844</x:v>
       </x:c>
       <x:c r="C143" s="1" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="D143" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E143" s="1" t="s">
-        <x:v>381</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="F143" s="1" t="s">
         <x:v>158</x:v>
@@ -11279,13 +11335,13 @@
         <x:v>46076.6465126505</x:v>
       </x:c>
       <x:c r="M143" s="1" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="R143" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
       <x:c r="S143" s="1" t="s">
-        <x:v>378</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="T143" s="1" t="n">
         <x:v>1</x:v>
@@ -11299,13 +11355,13 @@
         <x:v>35845</x:v>
       </x:c>
       <x:c r="C144" s="1" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="D144" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E144" s="1" t="s">
-        <x:v>382</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="F144" s="1" t="s">
         <x:v>158</x:v>
@@ -11326,13 +11382,13 @@
         <x:v>46076.6465126505</x:v>
       </x:c>
       <x:c r="M144" s="1" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="R144" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
       <x:c r="S144" s="1" t="s">
-        <x:v>378</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="T144" s="1" t="n">
         <x:v>1</x:v>
@@ -11346,13 +11402,13 @@
         <x:v>35846</x:v>
       </x:c>
       <x:c r="C145" s="1" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="D145" s="1" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E145" s="1" t="s">
-        <x:v>383</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="F145" s="1" t="s">
         <x:v>158</x:v>
@@ -11373,13 +11429,13 @@
         <x:v>46076.6465126505</x:v>
       </x:c>
       <x:c r="M145" s="1" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="R145" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
       <x:c r="S145" s="1" t="s">
-        <x:v>378</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="T145" s="1" t="n">
         <x:v>1</x:v>
@@ -11387,7 +11443,7 @@
     </x:row>
     <x:row r="146" spans="1:29">
       <x:c r="A146" s="4">
-        <x:v>46086.6571485764</x:v>
+        <x:v>46111.4966081019</x:v>
       </x:c>
       <x:c r="B146" s="1" t="n">
         <x:v>35888</x:v>
@@ -11396,19 +11452,19 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D146" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E146" s="1" t="s">
+        <x:v>383</x:v>
+      </x:c>
+      <x:c r="F146" s="1" t="s">
         <x:v>384</x:v>
-      </x:c>
-      <x:c r="F146" s="1" t="s">
-        <x:v>385</x:v>
       </x:c>
       <x:c r="G146" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H146" s="1" t="s">
-        <x:v>386</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="I146" s="1" t="n">
         <x:v>6</x:v>
@@ -11420,7 +11476,7 @@
         <x:v>46072.617799456</x:v>
       </x:c>
       <x:c r="M146" s="1" t="s">
-        <x:v>387</x:v>
+        <x:v>386</x:v>
       </x:c>
     </x:row>
     <x:row r="147" spans="1:29">
@@ -11434,19 +11490,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D147" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E147" s="1" t="s">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="F147" s="1" t="s">
         <x:v>388</x:v>
-      </x:c>
-      <x:c r="F147" s="1" t="s">
-        <x:v>389</x:v>
       </x:c>
       <x:c r="G147" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H147" s="1" t="s">
-        <x:v>390</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="I147" s="1" t="n">
         <x:v>12</x:v>
@@ -11461,7 +11517,7 @@
         <x:v>46086.6600798611</x:v>
       </x:c>
       <x:c r="M147" s="1" t="s">
-        <x:v>391</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="N147" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11479,7 +11535,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S147" s="1" t="s">
-        <x:v>392</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="T147" s="1" t="n">
         <x:v>23</x:v>
@@ -11505,19 +11561,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D148" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E148" s="1" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="F148" s="1" t="s">
         <x:v>393</x:v>
-      </x:c>
-      <x:c r="F148" s="1" t="s">
-        <x:v>394</x:v>
       </x:c>
       <x:c r="G148" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H148" s="1" t="s">
-        <x:v>395</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="I148" s="1" t="n">
         <x:v>12</x:v>
@@ -11532,7 +11588,7 @@
         <x:v>46086.6600798611</x:v>
       </x:c>
       <x:c r="M148" s="1" t="s">
-        <x:v>391</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="N148" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11550,7 +11606,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S148" s="1" t="s">
-        <x:v>392</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="T148" s="1" t="n">
         <x:v>23</x:v>
@@ -11567,7 +11623,7 @@
     </x:row>
     <x:row r="149" spans="1:29">
       <x:c r="A149" s="4">
-        <x:v>46086.6571485764</x:v>
+        <x:v>46111.4966081019</x:v>
       </x:c>
       <x:c r="B149" s="1" t="n">
         <x:v>35891</x:v>
@@ -11576,10 +11632,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D149" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E149" s="1" t="s">
-        <x:v>396</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="F149" s="1" t="s">
         <x:v>396</x:v>
@@ -11600,12 +11656,12 @@
         <x:v>46072.617799456</x:v>
       </x:c>
       <x:c r="M149" s="1" t="s">
-        <x:v>387</x:v>
+        <x:v>386</x:v>
       </x:c>
     </x:row>
     <x:row r="150" spans="1:29">
       <x:c r="A150" s="4">
-        <x:v>46086.6571485764</x:v>
+        <x:v>46111.4966081019</x:v>
       </x:c>
       <x:c r="B150" s="1" t="n">
         <x:v>35893</x:v>
@@ -11614,7 +11670,7 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D150" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E150" s="1" t="s">
         <x:v>398</x:v>
@@ -11638,12 +11694,12 @@
         <x:v>46072.617799456</x:v>
       </x:c>
       <x:c r="M150" s="1" t="s">
-        <x:v>387</x:v>
+        <x:v>386</x:v>
       </x:c>
     </x:row>
     <x:row r="151" spans="1:29">
       <x:c r="A151" s="4">
-        <x:v>46086.6557853356</x:v>
+        <x:v>46111.4595082523</x:v>
       </x:c>
       <x:c r="B151" s="1" t="n">
         <x:v>35894</x:v>
@@ -11658,7 +11714,7 @@
         <x:v>401</x:v>
       </x:c>
       <x:c r="F151" s="1" t="s">
-        <x:v>385</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="G151" s="1" t="s">
         <x:v>127</x:v>
@@ -11673,36 +11729,30 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L151" s="4">
-        <x:v>46072.6195613773</x:v>
+        <x:v>46107.609743669</x:v>
       </x:c>
       <x:c r="M151" s="1" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="R151" s="1" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="T151" s="1" t="n">
-        <x:v>21</x:v>
-      </x:c>
     </x:row>
     <x:row r="152" spans="1:29">
       <x:c r="A152" s="4">
-        <x:v>46086.6557853356</x:v>
+        <x:v>46099.715571794</x:v>
       </x:c>
       <x:c r="B152" s="1" t="n">
         <x:v>35895</x:v>
       </x:c>
       <x:c r="C152" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="D152" s="1" t="s">
         <x:v>321</x:v>
       </x:c>
       <x:c r="E152" s="1" t="s">
-        <x:v>404</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="F152" s="1" t="s">
-        <x:v>385</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="G152" s="1" t="s">
         <x:v>127</x:v>
@@ -11716,14 +11766,20 @@
       <x:c r="J152" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="K152" s="4">
+        <x:v>46099.7155716435</x:v>
+      </x:c>
       <x:c r="L152" s="4">
-        <x:v>46072.6195613773</x:v>
+        <x:v>46099.7155717245</x:v>
       </x:c>
       <x:c r="M152" s="1" t="s">
-        <x:v>403</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="R152" s="1" t="s">
-        <x:v>195</x:v>
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="S152" s="1" t="s">
+        <x:v>407</x:v>
       </x:c>
       <x:c r="T152" s="1" t="n">
         <x:v>21</x:v>
@@ -11731,28 +11787,28 @@
     </x:row>
     <x:row r="153" spans="1:29">
       <x:c r="A153" s="4">
-        <x:v>46086.6557853356</x:v>
+        <x:v>46107.610496794</x:v>
       </x:c>
       <x:c r="B153" s="1" t="n">
         <x:v>35896</x:v>
       </x:c>
       <x:c r="C153" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D153" s="1" t="s">
         <x:v>321</x:v>
       </x:c>
       <x:c r="E153" s="1" t="s">
-        <x:v>405</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="F153" s="1" t="s">
-        <x:v>406</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="G153" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H153" s="1" t="s">
-        <x:v>407</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="I153" s="1" t="n">
         <x:v>1</x:v>
@@ -11760,17 +11816,44 @@
       <x:c r="J153" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="K153" s="4">
+        <x:v>46098.4855049769</x:v>
+      </x:c>
       <x:c r="L153" s="4">
-        <x:v>46072.6195613773</x:v>
+        <x:v>46107.6101008102</x:v>
       </x:c>
       <x:c r="M153" s="1" t="s">
-        <x:v>403</x:v>
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="N153" s="4">
+        <x:v>46107.6101011227</x:v>
+      </x:c>
+      <x:c r="O153" s="1" t="s">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="P153" s="1" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="Q153" s="1" t="n">
+        <x:v>1318.185</x:v>
       </x:c>
       <x:c r="R153" s="1" t="s">
-        <x:v>195</x:v>
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="S153" s="1" t="s">
+        <x:v>414</x:v>
       </x:c>
       <x:c r="T153" s="1" t="n">
-        <x:v>21</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U153" s="1" t="s">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="V153" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W153" s="3">
+        <x:v>46115</x:v>
       </x:c>
     </x:row>
     <x:row r="154" spans="1:29">
@@ -11787,16 +11870,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E154" s="1" t="s">
-        <x:v>408</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="F154" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G154" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H154" s="1" t="s">
-        <x:v>409</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="I154" s="1" t="n">
         <x:v>4</x:v>
@@ -11811,7 +11894,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M154" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N154" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11829,7 +11912,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S154" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T154" s="1" t="n">
         <x:v>10</x:v>
@@ -11858,16 +11941,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E155" s="1" t="s">
-        <x:v>408</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="F155" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G155" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H155" s="1" t="s">
-        <x:v>412</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="I155" s="1" t="n">
         <x:v>4</x:v>
@@ -11882,7 +11965,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M155" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N155" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11900,7 +11983,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S155" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T155" s="1" t="n">
         <x:v>10</x:v>
@@ -11929,16 +12012,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E156" s="1" t="s">
-        <x:v>413</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="F156" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G156" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H156" s="1" t="s">
-        <x:v>414</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="I156" s="1" t="n">
         <x:v>4</x:v>
@@ -11953,7 +12036,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M156" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N156" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11971,7 +12054,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S156" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T156" s="1" t="n">
         <x:v>10</x:v>
@@ -12000,16 +12083,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E157" s="1" t="s">
-        <x:v>415</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="F157" s="1" t="s">
-        <x:v>416</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="G157" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H157" s="1" t="s">
-        <x:v>417</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="I157" s="1" t="n">
         <x:v>6</x:v>
@@ -12024,13 +12107,13 @@
         <x:v>46087.0783034375</x:v>
       </x:c>
       <x:c r="M157" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="N157" s="4">
         <x:v>46090.4474321412</x:v>
       </x:c>
       <x:c r="O157" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="P157" s="1" t="n">
         <x:v>8.5</x:v>
@@ -12039,16 +12122,16 @@
         <x:v>202.3935</x:v>
       </x:c>
       <x:c r="R157" s="1" t="s">
-        <x:v>420</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="S157" s="1" t="s">
-        <x:v>421</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="T157" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U157" s="1" t="s">
-        <x:v>422</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="V157" s="1" t="n">
         <x:v>6</x:v>
@@ -12071,16 +12154,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E158" s="1" t="s">
-        <x:v>423</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="F158" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G158" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H158" s="1" t="s">
-        <x:v>424</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="I158" s="1" t="n">
         <x:v>2</x:v>
@@ -12095,7 +12178,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M158" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N158" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12113,7 +12196,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S158" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T158" s="1" t="n">
         <x:v>10</x:v>
@@ -12136,22 +12219,22 @@
         <x:v>35902</x:v>
       </x:c>
       <x:c r="C159" s="1" t="s">
-        <x:v>425</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="D159" s="1" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E159" s="1" t="s">
-        <x:v>426</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="F159" s="1" t="s">
-        <x:v>385</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="G159" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H159" s="1" t="s">
-        <x:v>427</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="I159" s="1" t="n">
         <x:v>2</x:v>
@@ -12163,7 +12246,7 @@
         <x:v>46076.6827676736</x:v>
       </x:c>
       <x:c r="M159" s="1" t="s">
-        <x:v>428</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="R159" s="1" t="s">
         <x:v>195</x:v>
@@ -12183,16 +12266,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E160" s="1" t="s">
-        <x:v>429</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="F160" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G160" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H160" s="1" t="s">
-        <x:v>430</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="I160" s="1" t="n">
         <x:v>4</x:v>
@@ -12207,7 +12290,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M160" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N160" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12225,7 +12308,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S160" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T160" s="1" t="n">
         <x:v>10</x:v>
@@ -12254,16 +12337,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E161" s="1" t="s">
-        <x:v>431</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="F161" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G161" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H161" s="1" t="s">
-        <x:v>432</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I161" s="1" t="n">
         <x:v>4</x:v>
@@ -12278,7 +12361,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M161" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N161" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12296,7 +12379,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S161" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T161" s="1" t="n">
         <x:v>10</x:v>
@@ -12325,16 +12408,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E162" s="1" t="s">
-        <x:v>433</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="F162" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G162" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H162" s="1" t="s">
-        <x:v>434</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="I162" s="1" t="n">
         <x:v>4</x:v>
@@ -12349,7 +12432,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M162" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N162" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12367,7 +12450,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S162" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T162" s="1" t="n">
         <x:v>10</x:v>
@@ -12396,16 +12479,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E163" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="F163" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G163" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H163" s="1" t="s">
-        <x:v>436</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="I163" s="1" t="n">
         <x:v>1</x:v>
@@ -12420,7 +12503,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M163" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N163" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12438,7 +12521,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S163" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T163" s="1" t="n">
         <x:v>10</x:v>
@@ -12467,16 +12550,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E164" s="1" t="s">
-        <x:v>408</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="F164" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G164" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H164" s="1" t="s">
-        <x:v>437</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I164" s="1" t="n">
         <x:v>2</x:v>
@@ -12491,7 +12574,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M164" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N164" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12509,7 +12592,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S164" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T164" s="1" t="n">
         <x:v>10</x:v>
@@ -12538,16 +12621,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E165" s="1" t="s">
-        <x:v>413</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="F165" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G165" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H165" s="1" t="s">
-        <x:v>438</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="I165" s="1" t="n">
         <x:v>6</x:v>
@@ -12562,7 +12645,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M165" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N165" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12580,7 +12663,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S165" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T165" s="1" t="n">
         <x:v>10</x:v>
@@ -12609,16 +12692,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E166" s="1" t="s">
-        <x:v>439</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="F166" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G166" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H166" s="1" t="s">
-        <x:v>440</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="I166" s="1" t="n">
         <x:v>2</x:v>
@@ -12633,7 +12716,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M166" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N166" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12651,7 +12734,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S166" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T166" s="1" t="n">
         <x:v>10</x:v>
@@ -12680,16 +12763,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E167" s="1" t="s">
-        <x:v>415</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="F167" s="1" t="s">
-        <x:v>416</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="G167" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H167" s="1" t="s">
-        <x:v>441</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="I167" s="1" t="n">
         <x:v>2</x:v>
@@ -12704,13 +12787,13 @@
         <x:v>46087.0783034375</x:v>
       </x:c>
       <x:c r="M167" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="N167" s="4">
         <x:v>46090.4474321412</x:v>
       </x:c>
       <x:c r="O167" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="P167" s="1" t="n">
         <x:v>8.5</x:v>
@@ -12719,16 +12802,16 @@
         <x:v>67.4645</x:v>
       </x:c>
       <x:c r="R167" s="1" t="s">
-        <x:v>420</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="S167" s="1" t="s">
-        <x:v>421</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="T167" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U167" s="1" t="s">
-        <x:v>422</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="V167" s="1" t="n">
         <x:v>2</x:v>
@@ -12751,16 +12834,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E168" s="1" t="s">
-        <x:v>442</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="F168" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G168" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H168" s="1" t="s">
-        <x:v>443</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="I168" s="1" t="n">
         <x:v>8</x:v>
@@ -12775,7 +12858,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M168" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N168" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12793,7 +12876,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S168" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T168" s="1" t="n">
         <x:v>10</x:v>
@@ -12822,16 +12905,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E169" s="1" t="s">
-        <x:v>408</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="F169" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G169" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H169" s="1" t="s">
-        <x:v>444</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="I169" s="1" t="n">
         <x:v>2</x:v>
@@ -12846,7 +12929,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M169" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N169" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12864,7 +12947,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S169" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T169" s="1" t="n">
         <x:v>10</x:v>
@@ -12881,7 +12964,7 @@
     </x:row>
     <x:row r="170" spans="1:29">
       <x:c r="A170" s="4">
-        <x:v>46085.0734823264</x:v>
+        <x:v>46111.7199709144</x:v>
       </x:c>
       <x:c r="B170" s="1" t="n">
         <x:v>35913</x:v>
@@ -12893,16 +12976,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E170" s="1" t="s">
-        <x:v>445</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="F170" s="1" t="s">
-        <x:v>446</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="G170" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H170" s="1" t="s">
-        <x:v>447</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="I170" s="1" t="n">
         <x:v>1</x:v>
@@ -12911,10 +12994,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L170" s="4">
-        <x:v>46085.0733793634</x:v>
+        <x:v>46111.7199707986</x:v>
       </x:c>
       <x:c r="M170" s="1" t="s">
-        <x:v>448</x:v>
+        <x:v>454</x:v>
       </x:c>
     </x:row>
     <x:row r="171" spans="1:29">
@@ -12931,16 +13014,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E171" s="1" t="s">
-        <x:v>439</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="F171" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G171" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H171" s="1" t="s">
-        <x:v>449</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="I171" s="1" t="n">
         <x:v>4</x:v>
@@ -12955,7 +13038,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M171" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N171" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12973,7 +13056,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S171" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T171" s="1" t="n">
         <x:v>10</x:v>
@@ -13002,16 +13085,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E172" s="1" t="s">
-        <x:v>450</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="F172" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G172" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H172" s="1" t="s">
-        <x:v>451</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="I172" s="1" t="n">
         <x:v>1</x:v>
@@ -13026,7 +13109,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M172" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N172" s="4">
         <x:v>46090.4456414005</x:v>
@@ -13044,7 +13127,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S172" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T172" s="1" t="n">
         <x:v>10</x:v>
@@ -13073,16 +13156,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E173" s="1" t="s">
-        <x:v>452</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="F173" s="1" t="s">
-        <x:v>453</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="G173" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H173" s="1" t="s">
-        <x:v>454</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="I173" s="1" t="n">
         <x:v>1</x:v>
@@ -13097,13 +13180,13 @@
         <x:v>46090.4477212616</x:v>
       </x:c>
       <x:c r="M173" s="1" t="s">
-        <x:v>455</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="N173" s="4">
         <x:v>46090.447721412</x:v>
       </x:c>
       <x:c r="O173" s="1" t="s">
-        <x:v>456</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="P173" s="1" t="n">
         <x:v>885</x:v>
@@ -13112,16 +13195,16 @@
         <x:v>885</x:v>
       </x:c>
       <x:c r="R173" s="1" t="s">
-        <x:v>457</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="S173" s="1" t="s">
-        <x:v>458</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="T173" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U173" s="1" t="s">
-        <x:v>459</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="V173" s="1" t="n">
         <x:v>1</x:v>
@@ -13144,7 +13227,7 @@
         <x:v>138</x:v>
       </x:c>
       <x:c r="E174" s="1" t="s">
-        <x:v>460</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="F174" s="1" t="s">
         <x:v>51</x:v>
@@ -13165,13 +13248,13 @@
         <x:v>46092.627584375</x:v>
       </x:c>
       <x:c r="M174" s="1" t="s">
-        <x:v>461</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="N174" s="4">
         <x:v>46092.6275845255</x:v>
       </x:c>
       <x:c r="O174" s="1" t="s">
-        <x:v>462</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="P174" s="1" t="n">
         <x:v>66</x:v>
@@ -13183,13 +13266,13 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="S174" s="1" t="s">
-        <x:v>463</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="T174" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U174" s="1" t="s">
-        <x:v>464</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="V174" s="1" t="n">
         <x:v>2</x:v>
@@ -13200,28 +13283,28 @@
     </x:row>
     <x:row r="175" spans="1:29">
       <x:c r="A175" s="4">
-        <x:v>46093.004525081</x:v>
+        <x:v>46107.6118467593</x:v>
       </x:c>
       <x:c r="B175" s="1" t="n">
         <x:v>36279</x:v>
       </x:c>
       <x:c r="C175" s="1" t="s">
-        <x:v>465</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D175" s="1" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="E175" s="1" t="s">
-        <x:v>388</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="F175" s="1" t="s">
-        <x:v>466</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="G175" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H175" s="1" t="s">
-        <x:v>467</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="I175" s="1" t="n">
         <x:v>1</x:v>
@@ -13236,42 +13319,63 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M175" s="1" t="s">
-        <x:v>468</x:v>
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="N175" s="4">
+        <x:v>46107.6111298611</x:v>
+      </x:c>
+      <x:c r="O175" s="1" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="P175" s="1" t="n">
+        <x:v>137.84</x:v>
+      </x:c>
+      <x:c r="Q175" s="1" t="n">
+        <x:v>137.84</x:v>
       </x:c>
       <x:c r="R175" s="1" t="s">
         <x:v>195</x:v>
       </x:c>
       <x:c r="S175" s="1" t="s">
-        <x:v>469</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="T175" s="1" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U175" s="1" t="s">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="V175" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W175" s="3">
+        <x:v>46115</x:v>
       </x:c>
     </x:row>
     <x:row r="176" spans="1:29">
       <x:c r="A176" s="4">
-        <x:v>46093.004525081</x:v>
+        <x:v>46107.6118467593</x:v>
       </x:c>
       <x:c r="B176" s="1" t="n">
         <x:v>36280</x:v>
       </x:c>
       <x:c r="C176" s="1" t="s">
-        <x:v>465</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D176" s="1" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="E176" s="1" t="s">
-        <x:v>470</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="F176" s="1" t="s">
-        <x:v>466</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="G176" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H176" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="I176" s="1" t="n">
         <x:v>4</x:v>
@@ -13286,42 +13390,63 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M176" s="1" t="s">
-        <x:v>468</x:v>
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="N176" s="4">
+        <x:v>46107.6111298611</x:v>
+      </x:c>
+      <x:c r="O176" s="1" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="P176" s="1" t="n">
+        <x:v>1.02</x:v>
+      </x:c>
+      <x:c r="Q176" s="1" t="n">
+        <x:v>4.08</x:v>
       </x:c>
       <x:c r="R176" s="1" t="s">
         <x:v>195</x:v>
       </x:c>
       <x:c r="S176" s="1" t="s">
-        <x:v>469</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="T176" s="1" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U176" s="1" t="s">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="V176" s="1" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="W176" s="3">
+        <x:v>46115</x:v>
       </x:c>
     </x:row>
     <x:row r="177" spans="1:29">
       <x:c r="A177" s="4">
-        <x:v>46093.004525081</x:v>
+        <x:v>46107.6118467593</x:v>
       </x:c>
       <x:c r="B177" s="1" t="n">
         <x:v>36281</x:v>
       </x:c>
       <x:c r="C177" s="1" t="s">
-        <x:v>465</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D177" s="1" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="E177" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="F177" s="1" t="s">
-        <x:v>466</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="G177" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H177" s="1" t="s">
-        <x:v>473</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="I177" s="1" t="n">
         <x:v>4</x:v>
@@ -13336,21 +13461,42 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M177" s="1" t="s">
-        <x:v>468</x:v>
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="N177" s="4">
+        <x:v>46107.6111298611</x:v>
+      </x:c>
+      <x:c r="O177" s="1" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="P177" s="1" t="n">
+        <x:v>2.37</x:v>
+      </x:c>
+      <x:c r="Q177" s="1" t="n">
+        <x:v>9.48</x:v>
       </x:c>
       <x:c r="R177" s="1" t="s">
         <x:v>195</x:v>
       </x:c>
       <x:c r="S177" s="1" t="s">
-        <x:v>469</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="T177" s="1" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U177" s="1" t="s">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="V177" s="1" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="W177" s="3">
+        <x:v>46115</x:v>
       </x:c>
     </x:row>
     <x:row r="178" spans="1:29">
       <x:c r="A178" s="4">
-        <x:v>46093.0051498032</x:v>
+        <x:v>46097.6308056366</x:v>
       </x:c>
       <x:c r="B178" s="1" t="n">
         <x:v>36282</x:v>
@@ -13362,16 +13508,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E178" s="1" t="s">
-        <x:v>388</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="F178" s="1" t="s">
-        <x:v>474</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="G178" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H178" s="1" t="s">
-        <x:v>475</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="I178" s="1" t="n">
         <x:v>1</x:v>
@@ -13383,7 +13529,7 @@
         <x:v>46093.0051497338</x:v>
       </x:c>
       <x:c r="M178" s="1" t="s">
-        <x:v>476</x:v>
+        <x:v>483</x:v>
       </x:c>
     </x:row>
     <x:row r="179" spans="1:29">
@@ -13397,10 +13543,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D179" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E179" s="1" t="s">
-        <x:v>478</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="F179" s="1" t="s">
         <x:v>51</x:v>
@@ -13418,7 +13564,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M179" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="180" spans="1:29">
@@ -13432,10 +13578,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D180" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E180" s="1" t="s">
-        <x:v>480</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="F180" s="1" t="s">
         <x:v>64</x:v>
@@ -13453,7 +13599,7 @@
         <x:v>46085.4128305208</x:v>
       </x:c>
       <x:c r="M180" s="1" t="s">
-        <x:v>481</x:v>
+        <x:v>488</x:v>
       </x:c>
     </x:row>
     <x:row r="181" spans="1:29">
@@ -13467,10 +13613,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D181" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E181" s="1" t="s">
-        <x:v>482</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="F181" s="1" t="s">
         <x:v>51</x:v>
@@ -13488,7 +13634,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M181" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="182" spans="1:29">
@@ -13502,10 +13648,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D182" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E182" s="1" t="s">
-        <x:v>483</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="F182" s="1" t="s">
         <x:v>51</x:v>
@@ -13523,7 +13669,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M182" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="183" spans="1:29">
@@ -13537,10 +13683,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D183" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E183" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="F183" s="1" t="s">
         <x:v>51</x:v>
@@ -13558,7 +13704,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M183" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="184" spans="1:29">
@@ -13572,10 +13718,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D184" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E184" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="F184" s="1" t="s">
         <x:v>51</x:v>
@@ -13593,7 +13739,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M184" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="185" spans="1:29">
@@ -13607,10 +13753,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D185" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E185" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="F185" s="1" t="s">
         <x:v>51</x:v>
@@ -13628,7 +13774,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M185" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="186" spans="1:29">
@@ -13642,10 +13788,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D186" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E186" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F186" s="1" t="s">
         <x:v>51</x:v>
@@ -13663,7 +13809,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M186" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="187" spans="1:29">
@@ -13677,10 +13823,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D187" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E187" s="1" t="s">
-        <x:v>488</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="F187" s="1" t="s">
         <x:v>51</x:v>
@@ -13698,24 +13844,24 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M187" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="188" spans="1:29">
       <x:c r="A188" s="4">
-        <x:v>46086.6875060185</x:v>
+        <x:v>46111.7202197917</x:v>
       </x:c>
       <x:c r="B188" s="1" t="n">
         <x:v>36369</x:v>
       </x:c>
       <x:c r="C188" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D188" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E188" s="1" t="s">
-        <x:v>489</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="F188" s="1" t="s">
         <x:v>158</x:v>
@@ -13729,20 +13875,44 @@
       <x:c r="J188" s="1" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="K188" s="4">
+        <x:v>46111.6479773495</x:v>
+      </x:c>
       <x:c r="L188" s="4">
-        <x:v>46085.4131163542</x:v>
+        <x:v>46111.7201420139</x:v>
       </x:c>
       <x:c r="M188" s="1" t="s">
-        <x:v>490</x:v>
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="N188" s="4">
+        <x:v>46111.7201421644</x:v>
+      </x:c>
+      <x:c r="O188" s="1" t="s">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="P188" s="1" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="Q188" s="1" t="n">
+        <x:v>100</x:v>
       </x:c>
       <x:c r="R188" s="1" t="s">
         <x:v>161</x:v>
       </x:c>
       <x:c r="S188" s="1" t="s">
-        <x:v>491</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="T188" s="1" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="U188" s="1" t="s">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="V188" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W188" s="3">
+        <x:v>46126</x:v>
       </x:c>
     </x:row>
     <x:row r="189" spans="1:29">
@@ -13756,10 +13926,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D189" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E189" s="1" t="s">
-        <x:v>492</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="F189" s="1" t="s">
         <x:v>51</x:v>
@@ -13777,7 +13947,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M189" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="190" spans="1:29">
@@ -13791,10 +13961,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D190" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E190" s="1" t="s">
-        <x:v>493</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="F190" s="1" t="s">
         <x:v>51</x:v>
@@ -13812,7 +13982,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M190" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="191" spans="1:29">
@@ -13826,10 +13996,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D191" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E191" s="1" t="s">
-        <x:v>494</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="F191" s="1" t="s">
         <x:v>51</x:v>
@@ -13847,7 +14017,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M191" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="192" spans="1:29">
@@ -13861,19 +14031,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D192" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E192" s="1" t="s">
-        <x:v>495</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="F192" s="1" t="s">
-        <x:v>496</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="G192" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H192" s="1" t="s">
-        <x:v>497</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="I192" s="1" t="n">
         <x:v>2</x:v>
@@ -13888,7 +14058,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M192" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="N192" s="4">
         <x:v>46090.4456414005</x:v>
@@ -13906,7 +14076,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S192" s="1" t="s">
-        <x:v>499</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="T192" s="1" t="n">
         <x:v>1</x:v>
@@ -13932,19 +14102,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D193" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E193" s="1" t="s">
-        <x:v>500</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="F193" s="1" t="s">
-        <x:v>501</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="G193" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H193" s="1" t="s">
-        <x:v>502</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="I193" s="1" t="n">
         <x:v>2</x:v>
@@ -13959,7 +14129,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M193" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="N193" s="4">
         <x:v>46090.4456414005</x:v>
@@ -13977,7 +14147,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S193" s="1" t="s">
-        <x:v>499</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="T193" s="1" t="n">
         <x:v>1</x:v>
@@ -14003,10 +14173,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D194" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E194" s="1" t="s">
-        <x:v>503</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="F194" s="1" t="s">
         <x:v>222</x:v>
@@ -14015,7 +14185,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H194" s="1" t="s">
-        <x:v>504</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="I194" s="1" t="n">
         <x:v>2</x:v>
@@ -14030,7 +14200,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M194" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="N194" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14048,7 +14218,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S194" s="1" t="s">
-        <x:v>499</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="T194" s="1" t="n">
         <x:v>1</x:v>
@@ -14074,10 +14244,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D195" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E195" s="1" t="s">
-        <x:v>505</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="F195" s="1" t="s">
         <x:v>222</x:v>
@@ -14086,7 +14256,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H195" s="1" t="s">
-        <x:v>506</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="I195" s="1" t="n">
         <x:v>2</x:v>
@@ -14101,7 +14271,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M195" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="N195" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14119,7 +14289,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S195" s="1" t="s">
-        <x:v>499</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="T195" s="1" t="n">
         <x:v>1</x:v>
@@ -14145,7 +14315,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E196" s="1" t="s">
-        <x:v>507</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G196" s="1" t="s">
         <x:v>127</x:v>
@@ -14160,7 +14330,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M196" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="N196" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14178,7 +14348,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S196" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="T196" s="1" t="n">
         <x:v>10</x:v>
@@ -14204,10 +14374,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D197" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E197" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="F197" s="1" t="s">
         <x:v>64</x:v>
@@ -14225,7 +14395,7 @@
         <x:v>46086.7566555556</x:v>
       </x:c>
       <x:c r="M197" s="1" t="s">
-        <x:v>509</x:v>
+        <x:v>518</x:v>
       </x:c>
     </x:row>
     <x:row r="198" spans="1:29">
@@ -14239,7 +14409,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E198" s="1" t="s">
-        <x:v>510</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="G198" s="1" t="s">
         <x:v>127</x:v>
@@ -14254,7 +14424,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M198" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="N198" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14272,7 +14442,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S198" s="1" t="s">
-        <x:v>499</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="T198" s="1" t="n">
         <x:v>1</x:v>
@@ -14285,6 +14455,216 @@
       </x:c>
       <x:c r="W198" s="3">
         <x:v>46095</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" spans="1:29">
+      <x:c r="A199" s="4">
+        <x:v>46100.4842279745</x:v>
+      </x:c>
+      <x:c r="B199" s="1" t="n">
+        <x:v>37261</x:v>
+      </x:c>
+      <x:c r="C199" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D199" s="1" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="E199" s="1" t="s">
+        <x:v>521</x:v>
+      </x:c>
+      <x:c r="F199" s="1" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G199" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I199" s="1" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J199" s="1" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="L199" s="4">
+        <x:v>46098.5238698727</x:v>
+      </x:c>
+      <x:c r="M199" s="1" t="s">
+        <x:v>522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" spans="1:29">
+      <x:c r="A200" s="4">
+        <x:v>46100.4842279745</x:v>
+      </x:c>
+      <x:c r="B200" s="1" t="n">
+        <x:v>37262</x:v>
+      </x:c>
+      <x:c r="C200" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D200" s="1" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="E200" s="1" t="s">
+        <x:v>523</x:v>
+      </x:c>
+      <x:c r="F200" s="1" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G200" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I200" s="1" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J200" s="1" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L200" s="4">
+        <x:v>46098.5238698727</x:v>
+      </x:c>
+      <x:c r="M200" s="1" t="s">
+        <x:v>522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" spans="1:29">
+      <x:c r="A201" s="4">
+        <x:v>46100.4842279745</x:v>
+      </x:c>
+      <x:c r="B201" s="1" t="n">
+        <x:v>37265</x:v>
+      </x:c>
+      <x:c r="C201" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D201" s="1" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="E201" s="1" t="s">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="F201" s="1" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G201" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I201" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J201" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L201" s="4">
+        <x:v>46098.5238698727</x:v>
+      </x:c>
+      <x:c r="M201" s="1" t="s">
+        <x:v>522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" spans="1:29">
+      <x:c r="A202" s="4">
+        <x:v>46100.4842279745</x:v>
+      </x:c>
+      <x:c r="B202" s="1" t="n">
+        <x:v>37266</x:v>
+      </x:c>
+      <x:c r="C202" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D202" s="1" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="E202" s="1" t="s">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="F202" s="1" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G202" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I202" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J202" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L202" s="4">
+        <x:v>46098.5238698727</x:v>
+      </x:c>
+      <x:c r="M202" s="1" t="s">
+        <x:v>522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" spans="1:29">
+      <x:c r="A203" s="4">
+        <x:v>46100.4847336806</x:v>
+      </x:c>
+      <x:c r="B203" s="1" t="n">
+        <x:v>37412</x:v>
+      </x:c>
+      <x:c r="C203" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D203" s="1" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="E203" s="1" t="s">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="F203" s="1" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G203" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I203" s="1" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J203" s="1" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L203" s="4">
+        <x:v>46100.4729106481</x:v>
+      </x:c>
+      <x:c r="M203" s="1" t="s">
+        <x:v>527</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" spans="1:29">
+      <x:c r="A204" s="4">
+        <x:v>46100.4847336806</x:v>
+      </x:c>
+      <x:c r="B204" s="1" t="n">
+        <x:v>37413</x:v>
+      </x:c>
+      <x:c r="C204" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D204" s="1" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="E204" s="1" t="s">
+        <x:v>528</x:v>
+      </x:c>
+      <x:c r="F204" s="1" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G204" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I204" s="1" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J204" s="1" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="L204" s="4">
+        <x:v>46100.4729106481</x:v>
+      </x:c>
+      <x:c r="M204" s="1" t="s">
+        <x:v>527</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: add batch remark and fix floating bar scroll overlap
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="529">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="530">
   <x:si>
     <x:t>Document No</x:t>
   </x:si>
@@ -1266,7 +1266,7 @@
     <x:t>RFQ4134551</x:t>
   </x:si>
   <x:si>
-    <x:t>RFQ Reject</x:t>
+    <x:t>RFQ Approved</x:t>
   </x:si>
   <x:si>
     <x:t>clamp plate</x:t>
@@ -1360,6 +1360,9 @@
     <x:t xml:space="preserve">SSEBWZ16G-110
 【IAJ01-H16-L110】	
 </x:t>
+  </x:si>
+  <x:si>
+    <x:t>RFQ Reject</x:t>
   </x:si>
   <x:si>
     <x:t>Linear Guide Bearing</x:t>
@@ -11737,7 +11740,7 @@
     </x:row>
     <x:row r="152" spans="1:29">
       <x:c r="A152" s="4">
-        <x:v>46099.715571794</x:v>
+        <x:v>46114.6190235764</x:v>
       </x:c>
       <x:c r="B152" s="1" t="n">
         <x:v>35895</x:v>
@@ -11767,10 +11770,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="K152" s="4">
-        <x:v>46099.7155716435</x:v>
+        <x:v>46114.6190233796</x:v>
       </x:c>
       <x:c r="L152" s="4">
-        <x:v>46099.7155717245</x:v>
+        <x:v>46114.6190234954</x:v>
       </x:c>
       <x:c r="M152" s="1" t="s">
         <x:v>406</x:v>
@@ -12219,13 +12222,13 @@
         <x:v>35902</x:v>
       </x:c>
       <x:c r="C159" s="1" t="s">
-        <x:v>404</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D159" s="1" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E159" s="1" t="s">
-        <x:v>432</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="F159" s="1" t="s">
         <x:v>384</x:v>
@@ -12234,7 +12237,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H159" s="1" t="s">
-        <x:v>433</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="I159" s="1" t="n">
         <x:v>2</x:v>
@@ -12246,7 +12249,7 @@
         <x:v>46076.6827676736</x:v>
       </x:c>
       <x:c r="M159" s="1" t="s">
-        <x:v>434</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="R159" s="1" t="s">
         <x:v>195</x:v>
@@ -12266,7 +12269,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E160" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="F160" s="1" t="s">
         <x:v>393</x:v>
@@ -12275,7 +12278,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H160" s="1" t="s">
-        <x:v>436</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="I160" s="1" t="n">
         <x:v>4</x:v>
@@ -12337,7 +12340,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E161" s="1" t="s">
-        <x:v>437</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="F161" s="1" t="s">
         <x:v>393</x:v>
@@ -12346,7 +12349,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H161" s="1" t="s">
-        <x:v>438</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="I161" s="1" t="n">
         <x:v>4</x:v>
@@ -12408,7 +12411,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E162" s="1" t="s">
-        <x:v>439</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="F162" s="1" t="s">
         <x:v>393</x:v>
@@ -12417,7 +12420,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H162" s="1" t="s">
-        <x:v>440</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="I162" s="1" t="n">
         <x:v>4</x:v>
@@ -12479,7 +12482,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E163" s="1" t="s">
-        <x:v>441</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="F163" s="1" t="s">
         <x:v>393</x:v>
@@ -12488,7 +12491,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H163" s="1" t="s">
-        <x:v>442</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I163" s="1" t="n">
         <x:v>1</x:v>
@@ -12559,7 +12562,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H164" s="1" t="s">
-        <x:v>443</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="I164" s="1" t="n">
         <x:v>2</x:v>
@@ -12630,7 +12633,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H165" s="1" t="s">
-        <x:v>444</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="I165" s="1" t="n">
         <x:v>6</x:v>
@@ -12692,7 +12695,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E166" s="1" t="s">
-        <x:v>445</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="F166" s="1" t="s">
         <x:v>393</x:v>
@@ -12701,7 +12704,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H166" s="1" t="s">
-        <x:v>446</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="I166" s="1" t="n">
         <x:v>2</x:v>
@@ -12772,7 +12775,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H167" s="1" t="s">
-        <x:v>447</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="I167" s="1" t="n">
         <x:v>2</x:v>
@@ -12834,7 +12837,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E168" s="1" t="s">
-        <x:v>448</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="F168" s="1" t="s">
         <x:v>393</x:v>
@@ -12843,7 +12846,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H168" s="1" t="s">
-        <x:v>449</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="I168" s="1" t="n">
         <x:v>8</x:v>
@@ -12914,7 +12917,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H169" s="1" t="s">
-        <x:v>450</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="I169" s="1" t="n">
         <x:v>2</x:v>
@@ -12976,16 +12979,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E170" s="1" t="s">
-        <x:v>451</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="F170" s="1" t="s">
-        <x:v>452</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="G170" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H170" s="1" t="s">
-        <x:v>453</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="I170" s="1" t="n">
         <x:v>1</x:v>
@@ -12997,7 +13000,7 @@
         <x:v>46111.7199707986</x:v>
       </x:c>
       <x:c r="M170" s="1" t="s">
-        <x:v>454</x:v>
+        <x:v>455</x:v>
       </x:c>
     </x:row>
     <x:row r="171" spans="1:29">
@@ -13014,7 +13017,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E171" s="1" t="s">
-        <x:v>445</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="F171" s="1" t="s">
         <x:v>393</x:v>
@@ -13023,7 +13026,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H171" s="1" t="s">
-        <x:v>455</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="I171" s="1" t="n">
         <x:v>4</x:v>
@@ -13085,7 +13088,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E172" s="1" t="s">
-        <x:v>456</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="F172" s="1" t="s">
         <x:v>393</x:v>
@@ -13094,7 +13097,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H172" s="1" t="s">
-        <x:v>457</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="I172" s="1" t="n">
         <x:v>1</x:v>
@@ -13156,16 +13159,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E173" s="1" t="s">
-        <x:v>458</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F173" s="1" t="s">
-        <x:v>459</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G173" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H173" s="1" t="s">
-        <x:v>460</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="I173" s="1" t="n">
         <x:v>1</x:v>
@@ -13180,13 +13183,13 @@
         <x:v>46090.4477212616</x:v>
       </x:c>
       <x:c r="M173" s="1" t="s">
-        <x:v>461</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="N173" s="4">
         <x:v>46090.447721412</x:v>
       </x:c>
       <x:c r="O173" s="1" t="s">
-        <x:v>462</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="P173" s="1" t="n">
         <x:v>885</x:v>
@@ -13195,16 +13198,16 @@
         <x:v>885</x:v>
       </x:c>
       <x:c r="R173" s="1" t="s">
-        <x:v>463</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="S173" s="1" t="s">
-        <x:v>464</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="T173" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U173" s="1" t="s">
-        <x:v>465</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="V173" s="1" t="n">
         <x:v>1</x:v>
@@ -13227,7 +13230,7 @@
         <x:v>138</x:v>
       </x:c>
       <x:c r="E174" s="1" t="s">
-        <x:v>466</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="F174" s="1" t="s">
         <x:v>51</x:v>
@@ -13248,13 +13251,13 @@
         <x:v>46092.627584375</x:v>
       </x:c>
       <x:c r="M174" s="1" t="s">
-        <x:v>467</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="N174" s="4">
         <x:v>46092.6275845255</x:v>
       </x:c>
       <x:c r="O174" s="1" t="s">
-        <x:v>468</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="P174" s="1" t="n">
         <x:v>66</x:v>
@@ -13266,13 +13269,13 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="S174" s="1" t="s">
-        <x:v>469</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="T174" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U174" s="1" t="s">
-        <x:v>470</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="V174" s="1" t="n">
         <x:v>2</x:v>
@@ -13298,13 +13301,13 @@
         <x:v>387</x:v>
       </x:c>
       <x:c r="F175" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="G175" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H175" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="I175" s="1" t="n">
         <x:v>1</x:v>
@@ -13319,13 +13322,13 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M175" s="1" t="s">
-        <x:v>473</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="N175" s="4">
         <x:v>46107.6111298611</x:v>
       </x:c>
       <x:c r="O175" s="1" t="s">
-        <x:v>474</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="P175" s="1" t="n">
         <x:v>137.84</x:v>
@@ -13337,13 +13340,13 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="S175" s="1" t="s">
-        <x:v>475</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="T175" s="1" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="U175" s="1" t="s">
-        <x:v>476</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="V175" s="1" t="n">
         <x:v>1</x:v>
@@ -13366,16 +13369,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E176" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="F176" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="G176" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H176" s="1" t="s">
-        <x:v>478</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="I176" s="1" t="n">
         <x:v>4</x:v>
@@ -13390,13 +13393,13 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M176" s="1" t="s">
-        <x:v>473</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="N176" s="4">
         <x:v>46107.6111298611</x:v>
       </x:c>
       <x:c r="O176" s="1" t="s">
-        <x:v>474</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="P176" s="1" t="n">
         <x:v>1.02</x:v>
@@ -13408,13 +13411,13 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="S176" s="1" t="s">
-        <x:v>475</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="T176" s="1" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="U176" s="1" t="s">
-        <x:v>476</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="V176" s="1" t="n">
         <x:v>4</x:v>
@@ -13437,16 +13440,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E177" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="F177" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="G177" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H177" s="1" t="s">
-        <x:v>480</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="I177" s="1" t="n">
         <x:v>4</x:v>
@@ -13461,13 +13464,13 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M177" s="1" t="s">
-        <x:v>473</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="N177" s="4">
         <x:v>46107.6111298611</x:v>
       </x:c>
       <x:c r="O177" s="1" t="s">
-        <x:v>474</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="P177" s="1" t="n">
         <x:v>2.37</x:v>
@@ -13479,13 +13482,13 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="S177" s="1" t="s">
-        <x:v>475</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="T177" s="1" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="U177" s="1" t="s">
-        <x:v>476</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="V177" s="1" t="n">
         <x:v>4</x:v>
@@ -13511,13 +13514,13 @@
         <x:v>387</x:v>
       </x:c>
       <x:c r="F178" s="1" t="s">
-        <x:v>481</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="G178" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H178" s="1" t="s">
-        <x:v>482</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="I178" s="1" t="n">
         <x:v>1</x:v>
@@ -13529,7 +13532,7 @@
         <x:v>46093.0051497338</x:v>
       </x:c>
       <x:c r="M178" s="1" t="s">
-        <x:v>483</x:v>
+        <x:v>484</x:v>
       </x:c>
     </x:row>
     <x:row r="179" spans="1:29">
@@ -13543,10 +13546,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D179" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E179" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="F179" s="1" t="s">
         <x:v>51</x:v>
@@ -13564,7 +13567,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M179" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="180" spans="1:29">
@@ -13578,10 +13581,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D180" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E180" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="F180" s="1" t="s">
         <x:v>64</x:v>
@@ -13599,7 +13602,7 @@
         <x:v>46085.4128305208</x:v>
       </x:c>
       <x:c r="M180" s="1" t="s">
-        <x:v>488</x:v>
+        <x:v>489</x:v>
       </x:c>
     </x:row>
     <x:row r="181" spans="1:29">
@@ -13613,10 +13616,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D181" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E181" s="1" t="s">
-        <x:v>489</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="F181" s="1" t="s">
         <x:v>51</x:v>
@@ -13634,7 +13637,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M181" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="182" spans="1:29">
@@ -13648,10 +13651,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D182" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E182" s="1" t="s">
-        <x:v>490</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="F182" s="1" t="s">
         <x:v>51</x:v>
@@ -13669,7 +13672,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M182" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="183" spans="1:29">
@@ -13683,10 +13686,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D183" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E183" s="1" t="s">
-        <x:v>491</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="F183" s="1" t="s">
         <x:v>51</x:v>
@@ -13704,7 +13707,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M183" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="184" spans="1:29">
@@ -13718,10 +13721,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D184" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E184" s="1" t="s">
-        <x:v>492</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="F184" s="1" t="s">
         <x:v>51</x:v>
@@ -13739,7 +13742,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M184" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="185" spans="1:29">
@@ -13753,10 +13756,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D185" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E185" s="1" t="s">
-        <x:v>493</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F185" s="1" t="s">
         <x:v>51</x:v>
@@ -13774,7 +13777,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M185" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="186" spans="1:29">
@@ -13788,10 +13791,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D186" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E186" s="1" t="s">
-        <x:v>494</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="F186" s="1" t="s">
         <x:v>51</x:v>
@@ -13809,7 +13812,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M186" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="187" spans="1:29">
@@ -13823,10 +13826,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D187" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E187" s="1" t="s">
-        <x:v>495</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="F187" s="1" t="s">
         <x:v>51</x:v>
@@ -13844,7 +13847,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M187" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="188" spans="1:29">
@@ -13858,10 +13861,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D188" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E188" s="1" t="s">
-        <x:v>496</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="F188" s="1" t="s">
         <x:v>158</x:v>
@@ -13882,13 +13885,13 @@
         <x:v>46111.7201420139</x:v>
       </x:c>
       <x:c r="M188" s="1" t="s">
-        <x:v>497</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="N188" s="4">
         <x:v>46111.7201421644</x:v>
       </x:c>
       <x:c r="O188" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="P188" s="1" t="n">
         <x:v>50</x:v>
@@ -13900,13 +13903,13 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="S188" s="1" t="s">
-        <x:v>499</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="T188" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U188" s="1" t="s">
-        <x:v>500</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="V188" s="1" t="n">
         <x:v>2</x:v>
@@ -13926,10 +13929,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D189" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E189" s="1" t="s">
-        <x:v>501</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="F189" s="1" t="s">
         <x:v>51</x:v>
@@ -13947,7 +13950,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M189" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="190" spans="1:29">
@@ -13961,10 +13964,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D190" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E190" s="1" t="s">
-        <x:v>502</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="F190" s="1" t="s">
         <x:v>51</x:v>
@@ -13982,7 +13985,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M190" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="191" spans="1:29">
@@ -13996,10 +13999,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D191" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E191" s="1" t="s">
-        <x:v>503</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="F191" s="1" t="s">
         <x:v>51</x:v>
@@ -14017,7 +14020,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M191" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="192" spans="1:29">
@@ -14031,19 +14034,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D192" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E192" s="1" t="s">
-        <x:v>504</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="F192" s="1" t="s">
-        <x:v>505</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="G192" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H192" s="1" t="s">
-        <x:v>506</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="I192" s="1" t="n">
         <x:v>2</x:v>
@@ -14058,7 +14061,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M192" s="1" t="s">
-        <x:v>507</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="N192" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14076,7 +14079,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S192" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="T192" s="1" t="n">
         <x:v>1</x:v>
@@ -14102,19 +14105,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D193" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E193" s="1" t="s">
-        <x:v>509</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="F193" s="1" t="s">
-        <x:v>510</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G193" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H193" s="1" t="s">
-        <x:v>511</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I193" s="1" t="n">
         <x:v>2</x:v>
@@ -14129,7 +14132,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M193" s="1" t="s">
-        <x:v>507</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="N193" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14147,7 +14150,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S193" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="T193" s="1" t="n">
         <x:v>1</x:v>
@@ -14173,10 +14176,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D194" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E194" s="1" t="s">
-        <x:v>512</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="F194" s="1" t="s">
         <x:v>222</x:v>
@@ -14185,7 +14188,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H194" s="1" t="s">
-        <x:v>513</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="I194" s="1" t="n">
         <x:v>2</x:v>
@@ -14200,7 +14203,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M194" s="1" t="s">
-        <x:v>507</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="N194" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14218,7 +14221,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S194" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="T194" s="1" t="n">
         <x:v>1</x:v>
@@ -14244,10 +14247,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="D195" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E195" s="1" t="s">
-        <x:v>514</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="F195" s="1" t="s">
         <x:v>222</x:v>
@@ -14256,7 +14259,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H195" s="1" t="s">
-        <x:v>515</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="I195" s="1" t="n">
         <x:v>2</x:v>
@@ -14271,7 +14274,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M195" s="1" t="s">
-        <x:v>507</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="N195" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14289,7 +14292,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S195" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="T195" s="1" t="n">
         <x:v>1</x:v>
@@ -14315,7 +14318,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E196" s="1" t="s">
-        <x:v>516</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="G196" s="1" t="s">
         <x:v>127</x:v>
@@ -14374,10 +14377,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D197" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="E197" s="1" t="s">
-        <x:v>517</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="F197" s="1" t="s">
         <x:v>64</x:v>
@@ -14395,7 +14398,7 @@
         <x:v>46086.7566555556</x:v>
       </x:c>
       <x:c r="M197" s="1" t="s">
-        <x:v>518</x:v>
+        <x:v>519</x:v>
       </x:c>
     </x:row>
     <x:row r="198" spans="1:29">
@@ -14409,7 +14412,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E198" s="1" t="s">
-        <x:v>519</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="G198" s="1" t="s">
         <x:v>127</x:v>
@@ -14424,7 +14427,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M198" s="1" t="s">
-        <x:v>507</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="N198" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14442,7 +14445,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S198" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="T198" s="1" t="n">
         <x:v>1</x:v>
@@ -14468,10 +14471,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D199" s="1" t="s">
-        <x:v>520</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="E199" s="1" t="s">
-        <x:v>521</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="F199" s="1" t="s">
         <x:v>64</x:v>
@@ -14489,7 +14492,7 @@
         <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M199" s="1" t="s">
-        <x:v>522</x:v>
+        <x:v>523</x:v>
       </x:c>
     </x:row>
     <x:row r="200" spans="1:29">
@@ -14503,10 +14506,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D200" s="1" t="s">
-        <x:v>520</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="E200" s="1" t="s">
-        <x:v>523</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="F200" s="1" t="s">
         <x:v>64</x:v>
@@ -14524,7 +14527,7 @@
         <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M200" s="1" t="s">
-        <x:v>522</x:v>
+        <x:v>523</x:v>
       </x:c>
     </x:row>
     <x:row r="201" spans="1:29">
@@ -14538,10 +14541,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D201" s="1" t="s">
-        <x:v>520</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="E201" s="1" t="s">
-        <x:v>524</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="F201" s="1" t="s">
         <x:v>64</x:v>
@@ -14559,7 +14562,7 @@
         <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M201" s="1" t="s">
-        <x:v>522</x:v>
+        <x:v>523</x:v>
       </x:c>
     </x:row>
     <x:row r="202" spans="1:29">
@@ -14573,10 +14576,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D202" s="1" t="s">
-        <x:v>520</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="E202" s="1" t="s">
-        <x:v>525</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="F202" s="1" t="s">
         <x:v>64</x:v>
@@ -14594,7 +14597,7 @@
         <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M202" s="1" t="s">
-        <x:v>522</x:v>
+        <x:v>523</x:v>
       </x:c>
     </x:row>
     <x:row r="203" spans="1:29">
@@ -14608,10 +14611,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D203" s="1" t="s">
-        <x:v>520</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="E203" s="1" t="s">
-        <x:v>526</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="F203" s="1" t="s">
         <x:v>51</x:v>
@@ -14629,7 +14632,7 @@
         <x:v>46100.4729106481</x:v>
       </x:c>
       <x:c r="M203" s="1" t="s">
-        <x:v>527</x:v>
+        <x:v>528</x:v>
       </x:c>
     </x:row>
     <x:row r="204" spans="1:29">
@@ -14643,10 +14646,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D204" s="1" t="s">
-        <x:v>520</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="E204" s="1" t="s">
-        <x:v>528</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F204" s="1" t="s">
         <x:v>51</x:v>
@@ -14664,7 +14667,7 @@
         <x:v>46100.4729106481</x:v>
       </x:c>
       <x:c r="M204" s="1" t="s">
-        <x:v>527</x:v>
+        <x:v>528</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: add 'Other' status, exclude from stats, and enable status search/sort
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="530">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="533">
   <x:si>
     <x:t>Document No</x:t>
   </x:si>
@@ -1196,6 +1196,9 @@
     <x:t>OMR513-S1005A</x:t>
   </x:si>
   <x:si>
+    <x:t>PR Sent</x:t>
+  </x:si>
+  <x:si>
     <x:t>string wheel</x:t>
   </x:si>
   <x:si>
@@ -1205,7 +1208,14 @@
     <x:t>HBGP40-21</x:t>
   </x:si>
   <x:si>
-    <x:t>RFQ4129242</x:t>
+    <x:t>RFQ4136271</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PR5331101</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">https://internal.sophicauto.net/BOM/downloadFile/47659
+</x:t>
   </x:si>
   <x:si>
     <x:t>bearing</x:t>
@@ -1248,6 +1258,9 @@
     <x:t>A0-139452_EP01</x:t>
   </x:si>
   <x:si>
+    <x:t>RFQ4129242</x:t>
+  </x:si>
+  <x:si>
     <x:t>slipring</x:t>
   </x:si>
   <x:si>
@@ -1257,26 +1270,23 @@
     <x:t>LPC-06A</x:t>
   </x:si>
   <x:si>
-    <x:t>slider bearing</x:t>
-  </x:si>
-  <x:si>
-    <x:t>C-SX2RL24-L_b</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RFQ4134551</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RFQ Approved</x:t>
+    <x:t>RFQ4136261</x:t>
   </x:si>
   <x:si>
     <x:t>clamp plate</x:t>
   </x:si>
   <x:si>
     <x:t>RFQ4129252</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PR5330771</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://internal.sophicauto.net/BOM/downloadFile/45809
 </x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAPO26040033</x:t>
   </x:si>
   <x:si>
     <x:t>motor</x:t>
@@ -2075,7 +2085,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:AC204"/>
+  <x:dimension ref="A1:AC203"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="30" max="16384" width="9.140625" style="1" customWidth="1"/>
@@ -7394,7 +7404,7 @@
         <x:v>277</x:v>
       </x:c>
       <x:c r="T82" s="1" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U82" s="1" t="s">
         <x:v>278</x:v>
@@ -7465,7 +7475,7 @@
         <x:v>277</x:v>
       </x:c>
       <x:c r="T83" s="1" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U83" s="1" t="s">
         <x:v>278</x:v>
@@ -7607,7 +7617,7 @@
         <x:v>277</x:v>
       </x:c>
       <x:c r="T85" s="1" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U85" s="1" t="s">
         <x:v>292</x:v>
@@ -11446,28 +11456,28 @@
     </x:row>
     <x:row r="146" spans="1:29">
       <x:c r="A146" s="4">
-        <x:v>46111.4966081019</x:v>
+        <x:v>46115.7427043634</x:v>
       </x:c>
       <x:c r="B146" s="1" t="n">
         <x:v>35888</x:v>
       </x:c>
       <x:c r="C146" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="D146" s="1" t="s">
         <x:v>124</x:v>
       </x:c>
       <x:c r="E146" s="1" t="s">
-        <x:v>383</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="F146" s="1" t="s">
-        <x:v>384</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="G146" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H146" s="1" t="s">
-        <x:v>385</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="I146" s="1" t="n">
         <x:v>6</x:v>
@@ -11475,11 +11485,41 @@
       <x:c r="J146" s="1" t="n">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="K146" s="4">
+        <x:v>46115.6415685185</x:v>
+      </x:c>
       <x:c r="L146" s="4">
-        <x:v>46072.617799456</x:v>
+        <x:v>46115.7400868056</x:v>
       </x:c>
       <x:c r="M146" s="1" t="s">
-        <x:v>386</x:v>
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="N146" s="4">
+        <x:v>46115.7400869213</x:v>
+      </x:c>
+      <x:c r="O146" s="1" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="P146" s="1" t="n">
+        <x:v>126.51</x:v>
+      </x:c>
+      <x:c r="Q146" s="1" t="n">
+        <x:v>759.06</x:v>
+      </x:c>
+      <x:c r="R146" s="1" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="S146" s="1" t="s">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="T146" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V146" s="1" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="W146" s="4">
+        <x:v>46122.1666666667</x:v>
       </x:c>
     </x:row>
     <x:row r="147" spans="1:29">
@@ -11496,16 +11536,16 @@
         <x:v>124</x:v>
       </x:c>
       <x:c r="E147" s="1" t="s">
-        <x:v>387</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="F147" s="1" t="s">
-        <x:v>388</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="G147" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H147" s="1" t="s">
-        <x:v>389</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="I147" s="1" t="n">
         <x:v>12</x:v>
@@ -11520,7 +11560,7 @@
         <x:v>46086.6600798611</x:v>
       </x:c>
       <x:c r="M147" s="1" t="s">
-        <x:v>390</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="N147" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11538,7 +11578,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S147" s="1" t="s">
-        <x:v>391</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="T147" s="1" t="n">
         <x:v>23</x:v>
@@ -11567,16 +11607,16 @@
         <x:v>124</x:v>
       </x:c>
       <x:c r="E148" s="1" t="s">
-        <x:v>392</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="F148" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G148" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H148" s="1" t="s">
-        <x:v>394</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="I148" s="1" t="n">
         <x:v>12</x:v>
@@ -11591,7 +11631,7 @@
         <x:v>46086.6600798611</x:v>
       </x:c>
       <x:c r="M148" s="1" t="s">
-        <x:v>390</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="N148" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11609,7 +11649,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="S148" s="1" t="s">
-        <x:v>391</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="T148" s="1" t="n">
         <x:v>23</x:v>
@@ -11626,7 +11666,7 @@
     </x:row>
     <x:row r="149" spans="1:29">
       <x:c r="A149" s="4">
-        <x:v>46111.4966081019</x:v>
+        <x:v>46115.642734375</x:v>
       </x:c>
       <x:c r="B149" s="1" t="n">
         <x:v>35891</x:v>
@@ -11638,16 +11678,16 @@
         <x:v>124</x:v>
       </x:c>
       <x:c r="E149" s="1" t="s">
-        <x:v>395</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="F149" s="1" t="s">
-        <x:v>396</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="G149" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H149" s="1" t="s">
-        <x:v>397</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="I149" s="1" t="n">
         <x:v>1</x:v>
@@ -11659,12 +11699,15 @@
         <x:v>46072.617799456</x:v>
       </x:c>
       <x:c r="M149" s="1" t="s">
-        <x:v>386</x:v>
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="T149" s="1" t="s">
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="150" spans="1:29">
       <x:c r="A150" s="4">
-        <x:v>46111.4966081019</x:v>
+        <x:v>46115.6383925579</x:v>
       </x:c>
       <x:c r="B150" s="1" t="n">
         <x:v>35893</x:v>
@@ -11676,16 +11719,16 @@
         <x:v>124</x:v>
       </x:c>
       <x:c r="E150" s="1" t="s">
-        <x:v>398</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="F150" s="1" t="s">
-        <x:v>399</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="G150" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H150" s="1" t="s">
-        <x:v>400</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="I150" s="1" t="n">
         <x:v>2</x:v>
@@ -11694,74 +11737,107 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="L150" s="4">
-        <x:v>46072.617799456</x:v>
+        <x:v>46115.6381272338</x:v>
       </x:c>
       <x:c r="M150" s="1" t="s">
-        <x:v>386</x:v>
+        <x:v>405</x:v>
       </x:c>
     </x:row>
     <x:row r="151" spans="1:29">
       <x:c r="A151" s="4">
-        <x:v>46111.4595082523</x:v>
+        <x:v>46115.408791169</x:v>
       </x:c>
       <x:c r="B151" s="1" t="n">
-        <x:v>35894</x:v>
+        <x:v>35895</x:v>
       </x:c>
       <x:c r="C151" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D151" s="1" t="s">
         <x:v>321</x:v>
       </x:c>
       <x:c r="E151" s="1" t="s">
-        <x:v>401</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="F151" s="1" t="s">
-        <x:v>384</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="G151" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H151" s="1" t="s">
-        <x:v>402</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="I151" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J151" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K151" s="4">
+        <x:v>46114.6190233796</x:v>
       </x:c>
       <x:c r="L151" s="4">
-        <x:v>46107.609743669</x:v>
+        <x:v>46115.403372338</x:v>
       </x:c>
       <x:c r="M151" s="1" t="s">
-        <x:v>403</x:v>
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="N151" s="4">
+        <x:v>46115.4033724537</x:v>
+      </x:c>
+      <x:c r="O151" s="1" t="s">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="P151" s="1" t="n">
+        <x:v>3.38</x:v>
+      </x:c>
+      <x:c r="Q151" s="1" t="n">
+        <x:v>3.38</x:v>
+      </x:c>
+      <x:c r="R151" s="1" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="S151" s="1" t="s">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="T151" s="1" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="U151" s="1" t="s">
+        <x:v>410</x:v>
+      </x:c>
+      <x:c r="V151" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W151" s="4">
+        <x:v>46129.1666666667</x:v>
       </x:c>
     </x:row>
     <x:row r="152" spans="1:29">
       <x:c r="A152" s="4">
-        <x:v>46114.6190235764</x:v>
+        <x:v>46107.610496794</x:v>
       </x:c>
       <x:c r="B152" s="1" t="n">
-        <x:v>35895</x:v>
+        <x:v>35896</x:v>
       </x:c>
       <x:c r="C152" s="1" t="s">
-        <x:v>404</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D152" s="1" t="s">
         <x:v>321</x:v>
       </x:c>
       <x:c r="E152" s="1" t="s">
-        <x:v>405</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="F152" s="1" t="s">
-        <x:v>384</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="G152" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H152" s="1" t="s">
-        <x:v>304</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="I152" s="1" t="n">
         <x:v>1</x:v>
@@ -11770,93 +11846,114 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="K152" s="4">
-        <x:v>46114.6190233796</x:v>
+        <x:v>46098.4855049769</x:v>
       </x:c>
       <x:c r="L152" s="4">
-        <x:v>46114.6190234954</x:v>
+        <x:v>46107.6101008102</x:v>
       </x:c>
       <x:c r="M152" s="1" t="s">
-        <x:v>406</x:v>
+        <x:v>414</x:v>
+      </x:c>
+      <x:c r="N152" s="4">
+        <x:v>46107.6101011227</x:v>
+      </x:c>
+      <x:c r="O152" s="1" t="s">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="P152" s="1" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="Q152" s="1" t="n">
+        <x:v>1318.185</x:v>
       </x:c>
       <x:c r="R152" s="1" t="s">
-        <x:v>226</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="S152" s="1" t="s">
-        <x:v>407</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="T152" s="1" t="n">
-        <x:v>21</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U152" s="1" t="s">
+        <x:v>418</x:v>
+      </x:c>
+      <x:c r="V152" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W152" s="3">
+        <x:v>46115</x:v>
       </x:c>
     </x:row>
     <x:row r="153" spans="1:29">
       <x:c r="A153" s="4">
-        <x:v>46107.610496794</x:v>
+        <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B153" s="1" t="n">
-        <x:v>35896</x:v>
+        <x:v>35897</x:v>
       </x:c>
       <x:c r="C153" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
       <x:c r="D153" s="1" t="s">
-        <x:v>321</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E153" s="1" t="s">
-        <x:v>408</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F153" s="1" t="s">
-        <x:v>409</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G153" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H153" s="1" t="s">
-        <x:v>410</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="I153" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J153" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K153" s="4">
-        <x:v>46098.4855049769</x:v>
+        <x:v>46086.6518195255</x:v>
       </x:c>
       <x:c r="L153" s="4">
-        <x:v>46107.6101008102</x:v>
+        <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M153" s="1" t="s">
-        <x:v>411</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N153" s="4">
-        <x:v>46107.6101011227</x:v>
+        <x:v>46090.4456414005</x:v>
       </x:c>
       <x:c r="O153" s="1" t="s">
-        <x:v>412</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="P153" s="1" t="n">
-        <x:v>330</x:v>
+        <x:v>4.18</x:v>
       </x:c>
       <x:c r="Q153" s="1" t="n">
-        <x:v>1318.185</x:v>
+        <x:v>66.35332</x:v>
       </x:c>
       <x:c r="R153" s="1" t="s">
-        <x:v>413</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="S153" s="1" t="s">
-        <x:v>414</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T153" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="U153" s="1" t="s">
-        <x:v>415</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="V153" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W153" s="3">
-        <x:v>46115</x:v>
+        <x:v>46095</x:v>
       </x:c>
     </x:row>
     <x:row r="154" spans="1:29">
@@ -11864,7 +11961,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B154" s="1" t="n">
-        <x:v>35897</x:v>
+        <x:v>35898</x:v>
       </x:c>
       <x:c r="C154" s="1" t="s">
         <x:v>48</x:v>
@@ -11873,16 +11970,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E154" s="1" t="s">
-        <x:v>416</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F154" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G154" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H154" s="1" t="s">
-        <x:v>417</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="I154" s="1" t="n">
         <x:v>4</x:v>
@@ -11897,7 +11994,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M154" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N154" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11906,16 +12003,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P154" s="1" t="n">
-        <x:v>4.18</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="Q154" s="1" t="n">
-        <x:v>66.35332</x:v>
+        <x:v>80.9574</x:v>
       </x:c>
       <x:c r="R154" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S154" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T154" s="1" t="n">
         <x:v>10</x:v>
@@ -11935,7 +12032,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B155" s="1" t="n">
-        <x:v>35898</x:v>
+        <x:v>35899</x:v>
       </x:c>
       <x:c r="C155" s="1" t="s">
         <x:v>48</x:v>
@@ -11944,16 +12041,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E155" s="1" t="s">
-        <x:v>416</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="F155" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G155" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H155" s="1" t="s">
-        <x:v>420</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="I155" s="1" t="n">
         <x:v>4</x:v>
@@ -11968,7 +12065,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M155" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N155" s="4">
         <x:v>46090.4456414005</x:v>
@@ -11977,16 +12074,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P155" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="Q155" s="1" t="n">
-        <x:v>80.9574</x:v>
+        <x:v>3.1748</x:v>
       </x:c>
       <x:c r="R155" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S155" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T155" s="1" t="n">
         <x:v>10</x:v>
@@ -12003,10 +12100,10 @@
     </x:row>
     <x:row r="156" spans="1:29">
       <x:c r="A156" s="4">
-        <x:v>46090.4467435532</x:v>
+        <x:v>46090.4485225694</x:v>
       </x:c>
       <x:c r="B156" s="1" t="n">
-        <x:v>35899</x:v>
+        <x:v>35900</x:v>
       </x:c>
       <x:c r="C156" s="1" t="s">
         <x:v>48</x:v>
@@ -12015,69 +12112,69 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E156" s="1" t="s">
-        <x:v>421</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="F156" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="G156" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H156" s="1" t="s">
-        <x:v>422</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="I156" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J156" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K156" s="4">
-        <x:v>46086.6518195255</x:v>
+        <x:v>46087.078303206</x:v>
       </x:c>
       <x:c r="L156" s="4">
-        <x:v>46086.6518199421</x:v>
+        <x:v>46087.0783034375</x:v>
       </x:c>
       <x:c r="M156" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="N156" s="4">
-        <x:v>46090.4456414005</x:v>
+        <x:v>46090.4474321412</x:v>
       </x:c>
       <x:c r="O156" s="1" t="s">
-        <x:v>225</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="P156" s="1" t="n">
-        <x:v>0.2</x:v>
+        <x:v>8.5</x:v>
       </x:c>
       <x:c r="Q156" s="1" t="n">
-        <x:v>3.1748</x:v>
+        <x:v>202.3935</x:v>
       </x:c>
       <x:c r="R156" s="1" t="s">
-        <x:v>226</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="S156" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="T156" s="1" t="n">
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U156" s="1" t="s">
-        <x:v>228</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="V156" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W156" s="3">
-        <x:v>46095</x:v>
+        <x:v>46099</x:v>
       </x:c>
     </x:row>
     <x:row r="157" spans="1:29">
       <x:c r="A157" s="4">
-        <x:v>46090.4485225694</x:v>
+        <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B157" s="1" t="n">
-        <x:v>35900</x:v>
+        <x:v>35901</x:v>
       </x:c>
       <x:c r="C157" s="1" t="s">
         <x:v>48</x:v>
@@ -12086,87 +12183,87 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E157" s="1" t="s">
-        <x:v>423</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="F157" s="1" t="s">
-        <x:v>424</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G157" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H157" s="1" t="s">
-        <x:v>425</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="I157" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J157" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K157" s="4">
-        <x:v>46087.078303206</x:v>
+        <x:v>46086.6518195255</x:v>
       </x:c>
       <x:c r="L157" s="4">
-        <x:v>46087.0783034375</x:v>
+        <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M157" s="1" t="s">
-        <x:v>426</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N157" s="4">
-        <x:v>46090.4474321412</x:v>
+        <x:v>46090.4456414005</x:v>
       </x:c>
       <x:c r="O157" s="1" t="s">
-        <x:v>427</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="P157" s="1" t="n">
-        <x:v>8.5</x:v>
+        <x:v>35.63</x:v>
       </x:c>
       <x:c r="Q157" s="1" t="n">
-        <x:v>202.3935</x:v>
+        <x:v>282.79531</x:v>
       </x:c>
       <x:c r="R157" s="1" t="s">
-        <x:v>413</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="S157" s="1" t="s">
-        <x:v>428</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T157" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="U157" s="1" t="s">
-        <x:v>429</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="V157" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="W157" s="3">
-        <x:v>46099</x:v>
+        <x:v>46095</x:v>
       </x:c>
     </x:row>
     <x:row r="158" spans="1:29">
       <x:c r="A158" s="4">
-        <x:v>46090.4467435532</x:v>
+        <x:v>46086.6411116088</x:v>
       </x:c>
       <x:c r="B158" s="1" t="n">
-        <x:v>35901</x:v>
+        <x:v>35902</x:v>
       </x:c>
       <x:c r="C158" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="D158" s="1" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E158" s="1" t="s">
-        <x:v>430</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="F158" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="G158" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H158" s="1" t="s">
-        <x:v>431</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="I158" s="1" t="n">
         <x:v>2</x:v>
@@ -12174,85 +12271,85 @@
       <x:c r="J158" s="1" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K158" s="4">
-        <x:v>46086.6518195255</x:v>
-      </x:c>
       <x:c r="L158" s="4">
-        <x:v>46086.6518199421</x:v>
+        <x:v>46076.6827676736</x:v>
       </x:c>
       <x:c r="M158" s="1" t="s">
-        <x:v>418</x:v>
-      </x:c>
-      <x:c r="N158" s="4">
-        <x:v>46090.4456414005</x:v>
-      </x:c>
-      <x:c r="O158" s="1" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="P158" s="1" t="n">
-        <x:v>35.63</x:v>
-      </x:c>
-      <x:c r="Q158" s="1" t="n">
-        <x:v>282.79531</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="R158" s="1" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="S158" s="1" t="s">
-        <x:v>419</x:v>
-      </x:c>
-      <x:c r="T158" s="1" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="U158" s="1" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="V158" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="W158" s="3">
-        <x:v>46095</x:v>
+        <x:v>195</x:v>
       </x:c>
     </x:row>
     <x:row r="159" spans="1:29">
       <x:c r="A159" s="4">
-        <x:v>46086.6411116088</x:v>
+        <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B159" s="1" t="n">
-        <x:v>35902</x:v>
+        <x:v>35903</x:v>
       </x:c>
       <x:c r="C159" s="1" t="s">
-        <x:v>432</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D159" s="1" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E159" s="1" t="s">
-        <x:v>433</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="F159" s="1" t="s">
-        <x:v>384</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G159" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H159" s="1" t="s">
-        <x:v>434</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="I159" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J159" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K159" s="4">
+        <x:v>46086.6518195255</x:v>
       </x:c>
       <x:c r="L159" s="4">
-        <x:v>46076.6827676736</x:v>
+        <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M159" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="N159" s="4">
+        <x:v>46090.4456414005</x:v>
+      </x:c>
+      <x:c r="O159" s="1" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="P159" s="1" t="n">
+        <x:v>10.11</x:v>
+      </x:c>
+      <x:c r="Q159" s="1" t="n">
+        <x:v>160.48614</x:v>
       </x:c>
       <x:c r="R159" s="1" t="s">
-        <x:v>195</x:v>
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="S159" s="1" t="s">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="T159" s="1" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U159" s="1" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="V159" s="1" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="W159" s="3">
+        <x:v>46095</x:v>
       </x:c>
     </x:row>
     <x:row r="160" spans="1:29">
@@ -12260,7 +12357,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B160" s="1" t="n">
-        <x:v>35903</x:v>
+        <x:v>35904</x:v>
       </x:c>
       <x:c r="C160" s="1" t="s">
         <x:v>48</x:v>
@@ -12269,16 +12366,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E160" s="1" t="s">
-        <x:v>436</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="F160" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G160" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H160" s="1" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="I160" s="1" t="n">
         <x:v>4</x:v>
@@ -12293,7 +12390,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M160" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N160" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12302,16 +12399,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P160" s="1" t="n">
-        <x:v>10.11</x:v>
+        <x:v>0.82</x:v>
       </x:c>
       <x:c r="Q160" s="1" t="n">
-        <x:v>160.48614</x:v>
+        <x:v>13.01668</x:v>
       </x:c>
       <x:c r="R160" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S160" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T160" s="1" t="n">
         <x:v>10</x:v>
@@ -12331,7 +12428,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B161" s="1" t="n">
-        <x:v>35904</x:v>
+        <x:v>35905</x:v>
       </x:c>
       <x:c r="C161" s="1" t="s">
         <x:v>48</x:v>
@@ -12340,16 +12437,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E161" s="1" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="F161" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G161" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H161" s="1" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="I161" s="1" t="n">
         <x:v>4</x:v>
@@ -12364,7 +12461,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M161" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N161" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12373,16 +12470,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P161" s="1" t="n">
-        <x:v>0.82</x:v>
+        <x:v>0.15</x:v>
       </x:c>
       <x:c r="Q161" s="1" t="n">
-        <x:v>13.01668</x:v>
+        <x:v>2.3811</x:v>
       </x:c>
       <x:c r="R161" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S161" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T161" s="1" t="n">
         <x:v>10</x:v>
@@ -12402,7 +12499,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B162" s="1" t="n">
-        <x:v>35905</x:v>
+        <x:v>35906</x:v>
       </x:c>
       <x:c r="C162" s="1" t="s">
         <x:v>48</x:v>
@@ -12411,22 +12508,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E162" s="1" t="s">
-        <x:v>440</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="F162" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G162" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H162" s="1" t="s">
-        <x:v>441</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="I162" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J162" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K162" s="4">
         <x:v>46086.6518195255</x:v>
@@ -12435,7 +12532,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M162" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N162" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12444,16 +12541,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P162" s="1" t="n">
-        <x:v>0.15</x:v>
+        <x:v>3.65</x:v>
       </x:c>
       <x:c r="Q162" s="1" t="n">
-        <x:v>2.3811</x:v>
+        <x:v>14.485025</x:v>
       </x:c>
       <x:c r="R162" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S162" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T162" s="1" t="n">
         <x:v>10</x:v>
@@ -12462,7 +12559,7 @@
         <x:v>228</x:v>
       </x:c>
       <x:c r="V162" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W162" s="3">
         <x:v>46095</x:v>
@@ -12473,7 +12570,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B163" s="1" t="n">
-        <x:v>35906</x:v>
+        <x:v>35907</x:v>
       </x:c>
       <x:c r="C163" s="1" t="s">
         <x:v>48</x:v>
@@ -12482,22 +12579,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E163" s="1" t="s">
-        <x:v>442</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F163" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G163" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H163" s="1" t="s">
-        <x:v>443</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="I163" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J163" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K163" s="4">
         <x:v>46086.6518195255</x:v>
@@ -12506,7 +12603,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M163" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N163" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12515,16 +12612,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P163" s="1" t="n">
-        <x:v>3.65</x:v>
+        <x:v>6.75</x:v>
       </x:c>
       <x:c r="Q163" s="1" t="n">
-        <x:v>14.485025</x:v>
+        <x:v>53.57475</x:v>
       </x:c>
       <x:c r="R163" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S163" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T163" s="1" t="n">
         <x:v>10</x:v>
@@ -12533,7 +12630,7 @@
         <x:v>228</x:v>
       </x:c>
       <x:c r="V163" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="W163" s="3">
         <x:v>46095</x:v>
@@ -12544,7 +12641,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B164" s="1" t="n">
-        <x:v>35907</x:v>
+        <x:v>35908</x:v>
       </x:c>
       <x:c r="C164" s="1" t="s">
         <x:v>48</x:v>
@@ -12553,22 +12650,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E164" s="1" t="s">
-        <x:v>416</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="F164" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G164" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H164" s="1" t="s">
-        <x:v>444</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="I164" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J164" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K164" s="4">
         <x:v>46086.6518195255</x:v>
@@ -12577,7 +12674,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M164" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N164" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12586,16 +12683,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P164" s="1" t="n">
-        <x:v>6.75</x:v>
+        <x:v>0.16</x:v>
       </x:c>
       <x:c r="Q164" s="1" t="n">
-        <x:v>53.57475</x:v>
+        <x:v>3.80976</x:v>
       </x:c>
       <x:c r="R164" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S164" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T164" s="1" t="n">
         <x:v>10</x:v>
@@ -12604,7 +12701,7 @@
         <x:v>228</x:v>
       </x:c>
       <x:c r="V164" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W164" s="3">
         <x:v>46095</x:v>
@@ -12615,7 +12712,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B165" s="1" t="n">
-        <x:v>35908</x:v>
+        <x:v>35909</x:v>
       </x:c>
       <x:c r="C165" s="1" t="s">
         <x:v>48</x:v>
@@ -12624,22 +12721,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E165" s="1" t="s">
-        <x:v>421</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="F165" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G165" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H165" s="1" t="s">
-        <x:v>445</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="I165" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J165" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K165" s="4">
         <x:v>46086.6518195255</x:v>
@@ -12648,7 +12745,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M165" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N165" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12657,16 +12754,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P165" s="1" t="n">
-        <x:v>0.16</x:v>
+        <x:v>3.48</x:v>
       </x:c>
       <x:c r="Q165" s="1" t="n">
-        <x:v>3.80976</x:v>
+        <x:v>27.62076</x:v>
       </x:c>
       <x:c r="R165" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S165" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T165" s="1" t="n">
         <x:v>10</x:v>
@@ -12675,7 +12772,7 @@
         <x:v>228</x:v>
       </x:c>
       <x:c r="V165" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="W165" s="3">
         <x:v>46095</x:v>
@@ -12683,10 +12780,10 @@
     </x:row>
     <x:row r="166" spans="1:29">
       <x:c r="A166" s="4">
-        <x:v>46090.4467435532</x:v>
+        <x:v>46090.4485225694</x:v>
       </x:c>
       <x:c r="B166" s="1" t="n">
-        <x:v>35909</x:v>
+        <x:v>35910</x:v>
       </x:c>
       <x:c r="C166" s="1" t="s">
         <x:v>48</x:v>
@@ -12695,16 +12792,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E166" s="1" t="s">
-        <x:v>446</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="F166" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="G166" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H166" s="1" t="s">
-        <x:v>447</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="I166" s="1" t="n">
         <x:v>2</x:v>
@@ -12713,51 +12810,51 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="K166" s="4">
-        <x:v>46086.6518195255</x:v>
+        <x:v>46087.078303206</x:v>
       </x:c>
       <x:c r="L166" s="4">
-        <x:v>46086.6518199421</x:v>
+        <x:v>46087.0783034375</x:v>
       </x:c>
       <x:c r="M166" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="N166" s="4">
-        <x:v>46090.4456414005</x:v>
+        <x:v>46090.4474321412</x:v>
       </x:c>
       <x:c r="O166" s="1" t="s">
-        <x:v>225</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="P166" s="1" t="n">
-        <x:v>3.48</x:v>
+        <x:v>8.5</x:v>
       </x:c>
       <x:c r="Q166" s="1" t="n">
-        <x:v>27.62076</x:v>
+        <x:v>67.4645</x:v>
       </x:c>
       <x:c r="R166" s="1" t="s">
-        <x:v>226</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="S166" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="T166" s="1" t="n">
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U166" s="1" t="s">
-        <x:v>228</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="V166" s="1" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="W166" s="3">
-        <x:v>46095</x:v>
+        <x:v>46099</x:v>
       </x:c>
     </x:row>
     <x:row r="167" spans="1:29">
       <x:c r="A167" s="4">
-        <x:v>46090.4485225694</x:v>
+        <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B167" s="1" t="n">
-        <x:v>35910</x:v>
+        <x:v>35911</x:v>
       </x:c>
       <x:c r="C167" s="1" t="s">
         <x:v>48</x:v>
@@ -12766,61 +12863,61 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E167" s="1" t="s">
-        <x:v>423</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="F167" s="1" t="s">
-        <x:v>424</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G167" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H167" s="1" t="s">
-        <x:v>448</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="I167" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J167" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="K167" s="4">
-        <x:v>46087.078303206</x:v>
+        <x:v>46086.6518195255</x:v>
       </x:c>
       <x:c r="L167" s="4">
-        <x:v>46087.0783034375</x:v>
+        <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M167" s="1" t="s">
-        <x:v>426</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N167" s="4">
-        <x:v>46090.4474321412</x:v>
+        <x:v>46090.4456414005</x:v>
       </x:c>
       <x:c r="O167" s="1" t="s">
-        <x:v>427</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="P167" s="1" t="n">
-        <x:v>8.5</x:v>
+        <x:v>0.63</x:v>
       </x:c>
       <x:c r="Q167" s="1" t="n">
-        <x:v>67.4645</x:v>
+        <x:v>20.00124</x:v>
       </x:c>
       <x:c r="R167" s="1" t="s">
-        <x:v>413</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="S167" s="1" t="s">
-        <x:v>428</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T167" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="U167" s="1" t="s">
-        <x:v>429</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="V167" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W167" s="3">
-        <x:v>46099</x:v>
+        <x:v>46095</x:v>
       </x:c>
     </x:row>
     <x:row r="168" spans="1:29">
@@ -12828,7 +12925,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B168" s="1" t="n">
-        <x:v>35911</x:v>
+        <x:v>35912</x:v>
       </x:c>
       <x:c r="C168" s="1" t="s">
         <x:v>48</x:v>
@@ -12837,22 +12934,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E168" s="1" t="s">
-        <x:v>449</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F168" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G168" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H168" s="1" t="s">
-        <x:v>450</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="I168" s="1" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J168" s="1" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K168" s="4">
         <x:v>46086.6518195255</x:v>
@@ -12861,7 +12958,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M168" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N168" s="4">
         <x:v>46090.4456414005</x:v>
@@ -12870,16 +12967,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P168" s="1" t="n">
-        <x:v>0.63</x:v>
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="Q168" s="1" t="n">
-        <x:v>20.00124</x:v>
+        <x:v>13.88975</x:v>
       </x:c>
       <x:c r="R168" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S168" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T168" s="1" t="n">
         <x:v>10</x:v>
@@ -12888,7 +12985,7 @@
         <x:v>228</x:v>
       </x:c>
       <x:c r="V168" s="1" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="W168" s="3">
         <x:v>46095</x:v>
@@ -12896,111 +12993,111 @@
     </x:row>
     <x:row r="169" spans="1:29">
       <x:c r="A169" s="4">
-        <x:v>46090.4467435532</x:v>
+        <x:v>46111.7199709144</x:v>
       </x:c>
       <x:c r="B169" s="1" t="n">
-        <x:v>35912</x:v>
+        <x:v>35913</x:v>
       </x:c>
       <x:c r="C169" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D169" s="1" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E169" s="1" t="s">
-        <x:v>416</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="F169" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G169" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H169" s="1" t="s">
-        <x:v>451</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="I169" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J169" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K169" s="4">
-        <x:v>46086.6518195255</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L169" s="4">
-        <x:v>46086.6518199421</x:v>
+        <x:v>46111.7199707986</x:v>
       </x:c>
       <x:c r="M169" s="1" t="s">
-        <x:v>418</x:v>
-      </x:c>
-      <x:c r="N169" s="4">
-        <x:v>46090.4456414005</x:v>
-      </x:c>
-      <x:c r="O169" s="1" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="P169" s="1" t="n">
-        <x:v>1.75</x:v>
-      </x:c>
-      <x:c r="Q169" s="1" t="n">
-        <x:v>13.88975</x:v>
-      </x:c>
-      <x:c r="R169" s="1" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="S169" s="1" t="s">
-        <x:v>419</x:v>
-      </x:c>
-      <x:c r="T169" s="1" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="U169" s="1" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="V169" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="W169" s="3">
-        <x:v>46095</x:v>
+        <x:v>458</x:v>
       </x:c>
     </x:row>
     <x:row r="170" spans="1:29">
       <x:c r="A170" s="4">
-        <x:v>46111.7199709144</x:v>
+        <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B170" s="1" t="n">
-        <x:v>35913</x:v>
+        <x:v>35914</x:v>
       </x:c>
       <x:c r="C170" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D170" s="1" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E170" s="1" t="s">
-        <x:v>452</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="F170" s="1" t="s">
-        <x:v>453</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G170" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H170" s="1" t="s">
-        <x:v>454</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="I170" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J170" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K170" s="4">
+        <x:v>46086.6518195255</x:v>
       </x:c>
       <x:c r="L170" s="4">
-        <x:v>46111.7199707986</x:v>
+        <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M170" s="1" t="s">
-        <x:v>455</x:v>
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="N170" s="4">
+        <x:v>46090.4456414005</x:v>
+      </x:c>
+      <x:c r="O170" s="1" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="P170" s="1" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="Q170" s="1" t="n">
+        <x:v>58.7338</x:v>
+      </x:c>
+      <x:c r="R170" s="1" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="S170" s="1" t="s">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="T170" s="1" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U170" s="1" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="V170" s="1" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="W170" s="3">
+        <x:v>46095</x:v>
       </x:c>
     </x:row>
     <x:row r="171" spans="1:29">
@@ -13008,7 +13105,7 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B171" s="1" t="n">
-        <x:v>35914</x:v>
+        <x:v>35915</x:v>
       </x:c>
       <x:c r="C171" s="1" t="s">
         <x:v>48</x:v>
@@ -13017,22 +13114,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E171" s="1" t="s">
-        <x:v>446</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="F171" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G171" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H171" s="1" t="s">
-        <x:v>456</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="I171" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J171" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K171" s="4">
         <x:v>46086.6518195255</x:v>
@@ -13041,7 +13138,7 @@
         <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M171" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N171" s="4">
         <x:v>46090.4456414005</x:v>
@@ -13050,16 +13147,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P171" s="1" t="n">
-        <x:v>3.7</x:v>
+        <x:v>5.86</x:v>
       </x:c>
       <x:c r="Q171" s="1" t="n">
-        <x:v>58.7338</x:v>
+        <x:v>23.25541</x:v>
       </x:c>
       <x:c r="R171" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S171" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T171" s="1" t="n">
         <x:v>10</x:v>
@@ -13068,7 +13165,7 @@
         <x:v>228</x:v>
       </x:c>
       <x:c r="V171" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W171" s="3">
         <x:v>46095</x:v>
@@ -13076,10 +13173,10 @@
     </x:row>
     <x:row r="172" spans="1:29">
       <x:c r="A172" s="4">
-        <x:v>46090.4467435532</x:v>
+        <x:v>46090.447941169</x:v>
       </x:c>
       <x:c r="B172" s="1" t="n">
-        <x:v>35915</x:v>
+        <x:v>35916</x:v>
       </x:c>
       <x:c r="C172" s="1" t="s">
         <x:v>48</x:v>
@@ -13088,16 +13185,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E172" s="1" t="s">
-        <x:v>457</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="F172" s="1" t="s">
-        <x:v>393</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="G172" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H172" s="1" t="s">
-        <x:v>458</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="I172" s="1" t="n">
         <x:v>1</x:v>
@@ -13106,182 +13203,182 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="K172" s="4">
-        <x:v>46086.6518195255</x:v>
+        <x:v>46085.6136977199</x:v>
       </x:c>
       <x:c r="L172" s="4">
-        <x:v>46086.6518199421</x:v>
+        <x:v>46090.4477212616</x:v>
       </x:c>
       <x:c r="M172" s="1" t="s">
-        <x:v>418</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="N172" s="4">
-        <x:v>46090.4456414005</x:v>
+        <x:v>46090.447721412</x:v>
       </x:c>
       <x:c r="O172" s="1" t="s">
-        <x:v>225</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="P172" s="1" t="n">
-        <x:v>5.86</x:v>
+        <x:v>885</x:v>
       </x:c>
       <x:c r="Q172" s="1" t="n">
-        <x:v>23.25541</x:v>
+        <x:v>885</x:v>
       </x:c>
       <x:c r="R172" s="1" t="s">
-        <x:v>226</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="S172" s="1" t="s">
-        <x:v>419</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="T172" s="1" t="n">
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U172" s="1" t="s">
-        <x:v>228</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="V172" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="W172" s="3">
-        <x:v>46095</x:v>
+        <x:v>46113</x:v>
       </x:c>
     </x:row>
     <x:row r="173" spans="1:29">
       <x:c r="A173" s="4">
-        <x:v>46090.447941169</x:v>
+        <x:v>46092.6276936343</x:v>
       </x:c>
       <x:c r="B173" s="1" t="n">
-        <x:v>35916</x:v>
+        <x:v>36010</x:v>
       </x:c>
       <x:c r="C173" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
       <x:c r="D173" s="1" t="s">
-        <x:v>80</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="E173" s="1" t="s">
-        <x:v>459</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="F173" s="1" t="s">
-        <x:v>460</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G173" s="1" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="H173" s="1" t="s">
-        <x:v>461</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="I173" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J173" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K173" s="4">
-        <x:v>46085.6136977199</x:v>
+        <x:v>46092.6231591088</x:v>
       </x:c>
       <x:c r="L173" s="4">
-        <x:v>46090.4477212616</x:v>
+        <x:v>46092.627584375</x:v>
       </x:c>
       <x:c r="M173" s="1" t="s">
-        <x:v>462</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="N173" s="4">
-        <x:v>46090.447721412</x:v>
+        <x:v>46092.6275845255</x:v>
       </x:c>
       <x:c r="O173" s="1" t="s">
-        <x:v>463</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="P173" s="1" t="n">
-        <x:v>885</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="Q173" s="1" t="n">
-        <x:v>885</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="R173" s="1" t="s">
-        <x:v>464</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="S173" s="1" t="s">
-        <x:v>465</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="T173" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="U173" s="1" t="s">
-        <x:v>466</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="V173" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="W173" s="3">
-        <x:v>46113</x:v>
+        <x:v>46094</x:v>
       </x:c>
     </x:row>
     <x:row r="174" spans="1:29">
       <x:c r="A174" s="4">
-        <x:v>46092.6276936343</x:v>
+        <x:v>46107.6118467593</x:v>
       </x:c>
       <x:c r="B174" s="1" t="n">
-        <x:v>36010</x:v>
+        <x:v>36279</x:v>
       </x:c>
       <x:c r="C174" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
       <x:c r="D174" s="1" t="s">
-        <x:v>138</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E174" s="1" t="s">
-        <x:v>467</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="F174" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="G174" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="H174" s="1" t="s">
+        <x:v>476</x:v>
       </x:c>
       <x:c r="I174" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J174" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K174" s="4">
-        <x:v>46092.6231591088</x:v>
+        <x:v>46093.0045248843</x:v>
       </x:c>
       <x:c r="L174" s="4">
-        <x:v>46092.627584375</x:v>
+        <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M174" s="1" t="s">
-        <x:v>468</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="N174" s="4">
-        <x:v>46092.6275845255</x:v>
+        <x:v>46107.6111298611</x:v>
       </x:c>
       <x:c r="O174" s="1" t="s">
-        <x:v>469</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="P174" s="1" t="n">
-        <x:v>66</x:v>
+        <x:v>137.84</x:v>
       </x:c>
       <x:c r="Q174" s="1" t="n">
-        <x:v>132</x:v>
+        <x:v>137.84</x:v>
       </x:c>
       <x:c r="R174" s="1" t="s">
-        <x:v>147</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="S174" s="1" t="s">
-        <x:v>470</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="T174" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="U174" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="V174" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W174" s="3">
-        <x:v>46094</x:v>
+        <x:v>46115</x:v>
       </x:c>
     </x:row>
     <x:row r="175" spans="1:29">
@@ -13289,7 +13386,7 @@
         <x:v>46107.6118467593</x:v>
       </x:c>
       <x:c r="B175" s="1" t="n">
-        <x:v>36279</x:v>
+        <x:v>36280</x:v>
       </x:c>
       <x:c r="C175" s="1" t="s">
         <x:v>48</x:v>
@@ -13298,22 +13395,22 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E175" s="1" t="s">
-        <x:v>387</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="F175" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="G175" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H175" s="1" t="s">
-        <x:v>473</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="I175" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J175" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K175" s="4">
         <x:v>46093.0045248843</x:v>
@@ -13322,34 +13419,34 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M175" s="1" t="s">
-        <x:v>474</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="N175" s="4">
         <x:v>46107.6111298611</x:v>
       </x:c>
       <x:c r="O175" s="1" t="s">
-        <x:v>475</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="P175" s="1" t="n">
-        <x:v>137.84</x:v>
+        <x:v>1.02</x:v>
       </x:c>
       <x:c r="Q175" s="1" t="n">
-        <x:v>137.84</x:v>
+        <x:v>4.08</x:v>
       </x:c>
       <x:c r="R175" s="1" t="s">
         <x:v>195</x:v>
       </x:c>
       <x:c r="S175" s="1" t="s">
-        <x:v>476</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="T175" s="1" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="U175" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="V175" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W175" s="3">
         <x:v>46115</x:v>
@@ -13360,7 +13457,7 @@
         <x:v>46107.6118467593</x:v>
       </x:c>
       <x:c r="B176" s="1" t="n">
-        <x:v>36280</x:v>
+        <x:v>36281</x:v>
       </x:c>
       <x:c r="C176" s="1" t="s">
         <x:v>48</x:v>
@@ -13369,16 +13466,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E176" s="1" t="s">
-        <x:v>478</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="F176" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="G176" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H176" s="1" t="s">
-        <x:v>479</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="I176" s="1" t="n">
         <x:v>4</x:v>
@@ -13393,31 +13490,31 @@
         <x:v>46093.0045250347</x:v>
       </x:c>
       <x:c r="M176" s="1" t="s">
-        <x:v>474</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="N176" s="4">
         <x:v>46107.6111298611</x:v>
       </x:c>
       <x:c r="O176" s="1" t="s">
-        <x:v>475</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="P176" s="1" t="n">
-        <x:v>1.02</x:v>
+        <x:v>2.37</x:v>
       </x:c>
       <x:c r="Q176" s="1" t="n">
-        <x:v>4.08</x:v>
+        <x:v>9.48</x:v>
       </x:c>
       <x:c r="R176" s="1" t="s">
         <x:v>195</x:v>
       </x:c>
       <x:c r="S176" s="1" t="s">
-        <x:v>476</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="T176" s="1" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="U176" s="1" t="s">
-        <x:v>477</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="V176" s="1" t="n">
         <x:v>4</x:v>
@@ -13428,181 +13525,145 @@
     </x:row>
     <x:row r="177" spans="1:29">
       <x:c r="A177" s="4">
-        <x:v>46107.6118467593</x:v>
+        <x:v>46097.6308056366</x:v>
       </x:c>
       <x:c r="B177" s="1" t="n">
-        <x:v>36281</x:v>
+        <x:v>36282</x:v>
       </x:c>
       <x:c r="C177" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D177" s="1" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="E177" s="1" t="s">
-        <x:v>480</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="F177" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="G177" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H177" s="1" t="s">
-        <x:v>481</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="I177" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J177" s="1" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="K177" s="4">
-        <x:v>46093.0045248843</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L177" s="4">
-        <x:v>46093.0045250347</x:v>
+        <x:v>46093.0051497338</x:v>
       </x:c>
       <x:c r="M177" s="1" t="s">
-        <x:v>474</x:v>
-      </x:c>
-      <x:c r="N177" s="4">
-        <x:v>46107.6111298611</x:v>
-      </x:c>
-      <x:c r="O177" s="1" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="P177" s="1" t="n">
-        <x:v>2.37</x:v>
-      </x:c>
-      <x:c r="Q177" s="1" t="n">
-        <x:v>9.48</x:v>
-      </x:c>
-      <x:c r="R177" s="1" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="S177" s="1" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="T177" s="1" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="U177" s="1" t="s">
-        <x:v>477</x:v>
-      </x:c>
-      <x:c r="V177" s="1" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="W177" s="3">
-        <x:v>46115</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="178" spans="1:29">
       <x:c r="A178" s="4">
-        <x:v>46097.6308056366</x:v>
+        <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B178" s="1" t="n">
-        <x:v>36282</x:v>
+        <x:v>36360</x:v>
       </x:c>
       <x:c r="C178" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D178" s="1" t="s">
-        <x:v>49</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E178" s="1" t="s">
-        <x:v>387</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="F178" s="1" t="s">
-        <x:v>482</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G178" s="1" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="H178" s="1" t="s">
-        <x:v>483</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="I178" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J178" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L178" s="4">
-        <x:v>46093.0051497338</x:v>
+        <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M178" s="1" t="s">
-        <x:v>484</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="179" spans="1:29">
       <x:c r="A179" s="4">
-        <x:v>46085.4171919792</x:v>
+        <x:v>46085.4166482292</x:v>
       </x:c>
       <x:c r="B179" s="1" t="n">
-        <x:v>36360</x:v>
+        <x:v>36361</x:v>
       </x:c>
       <x:c r="C179" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D179" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E179" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="F179" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="G179" s="1" t="s">
         <x:v>52</x:v>
       </x:c>
       <x:c r="I179" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J179" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L179" s="4">
-        <x:v>46085.4124951389</x:v>
+        <x:v>46085.4128305208</x:v>
       </x:c>
       <x:c r="M179" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>492</x:v>
       </x:c>
     </x:row>
     <x:row r="180" spans="1:29">
       <x:c r="A180" s="4">
-        <x:v>46085.4166482292</x:v>
+        <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B180" s="1" t="n">
-        <x:v>36361</x:v>
+        <x:v>36362</x:v>
       </x:c>
       <x:c r="C180" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D180" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E180" s="1" t="s">
-        <x:v>488</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="F180" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G180" s="1" t="s">
         <x:v>52</x:v>
       </x:c>
       <x:c r="I180" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J180" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L180" s="4">
-        <x:v>46085.4128305208</x:v>
+        <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M180" s="1" t="s">
-        <x:v>489</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="181" spans="1:29">
@@ -13610,16 +13671,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B181" s="1" t="n">
-        <x:v>36362</x:v>
+        <x:v>36363</x:v>
       </x:c>
       <x:c r="C181" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D181" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E181" s="1" t="s">
-        <x:v>490</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F181" s="1" t="s">
         <x:v>51</x:v>
@@ -13637,7 +13698,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M181" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="182" spans="1:29">
@@ -13645,16 +13706,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B182" s="1" t="n">
-        <x:v>36363</x:v>
+        <x:v>36364</x:v>
       </x:c>
       <x:c r="C182" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D182" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E182" s="1" t="s">
-        <x:v>491</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="F182" s="1" t="s">
         <x:v>51</x:v>
@@ -13663,16 +13724,16 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="I182" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J182" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L182" s="4">
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M182" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="183" spans="1:29">
@@ -13680,16 +13741,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B183" s="1" t="n">
-        <x:v>36364</x:v>
+        <x:v>36365</x:v>
       </x:c>
       <x:c r="C183" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D183" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E183" s="1" t="s">
-        <x:v>492</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="F183" s="1" t="s">
         <x:v>51</x:v>
@@ -13698,16 +13759,16 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="I183" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J183" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L183" s="4">
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M183" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="184" spans="1:29">
@@ -13715,16 +13776,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B184" s="1" t="n">
-        <x:v>36365</x:v>
+        <x:v>36366</x:v>
       </x:c>
       <x:c r="C184" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D184" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E184" s="1" t="s">
-        <x:v>493</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="F184" s="1" t="s">
         <x:v>51</x:v>
@@ -13742,7 +13803,7 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M184" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="185" spans="1:29">
@@ -13750,16 +13811,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B185" s="1" t="n">
-        <x:v>36366</x:v>
+        <x:v>36367</x:v>
       </x:c>
       <x:c r="C185" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D185" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E185" s="1" t="s">
-        <x:v>494</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="F185" s="1" t="s">
         <x:v>51</x:v>
@@ -13768,16 +13829,16 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="I185" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J185" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L185" s="4">
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M185" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="186" spans="1:29">
@@ -13785,16 +13846,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B186" s="1" t="n">
-        <x:v>36367</x:v>
+        <x:v>36368</x:v>
       </x:c>
       <x:c r="C186" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D186" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E186" s="1" t="s">
-        <x:v>495</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="F186" s="1" t="s">
         <x:v>51</x:v>
@@ -13812,110 +13873,110 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M186" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="187" spans="1:29">
       <x:c r="A187" s="4">
-        <x:v>46085.4171919792</x:v>
+        <x:v>46111.7202197917</x:v>
       </x:c>
       <x:c r="B187" s="1" t="n">
-        <x:v>36368</x:v>
+        <x:v>36369</x:v>
       </x:c>
       <x:c r="C187" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D187" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E187" s="1" t="s">
-        <x:v>496</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="F187" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="G187" s="1" t="s">
         <x:v>52</x:v>
       </x:c>
       <x:c r="I187" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J187" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K187" s="4">
+        <x:v>46111.6479773495</x:v>
       </x:c>
       <x:c r="L187" s="4">
-        <x:v>46085.4124951389</x:v>
+        <x:v>46111.7201420139</x:v>
       </x:c>
       <x:c r="M187" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="N187" s="4">
+        <x:v>46111.7201421644</x:v>
+      </x:c>
+      <x:c r="O187" s="1" t="s">
+        <x:v>502</x:v>
+      </x:c>
+      <x:c r="P187" s="1" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="Q187" s="1" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="R187" s="1" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="S187" s="1" t="s">
+        <x:v>503</x:v>
+      </x:c>
+      <x:c r="T187" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U187" s="1" t="s">
+        <x:v>504</x:v>
+      </x:c>
+      <x:c r="V187" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W187" s="3">
+        <x:v>46126</x:v>
       </x:c>
     </x:row>
     <x:row r="188" spans="1:29">
       <x:c r="A188" s="4">
-        <x:v>46111.7202197917</x:v>
+        <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B188" s="1" t="n">
-        <x:v>36369</x:v>
+        <x:v>36370</x:v>
       </x:c>
       <x:c r="C188" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D188" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E188" s="1" t="s">
-        <x:v>497</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="F188" s="1" t="s">
-        <x:v>158</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G188" s="1" t="s">
         <x:v>52</x:v>
       </x:c>
       <x:c r="I188" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J188" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K188" s="4">
-        <x:v>46111.6479773495</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L188" s="4">
-        <x:v>46111.7201420139</x:v>
+        <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M188" s="1" t="s">
-        <x:v>498</x:v>
-      </x:c>
-      <x:c r="N188" s="4">
-        <x:v>46111.7201421644</x:v>
-      </x:c>
-      <x:c r="O188" s="1" t="s">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="P188" s="1" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="Q188" s="1" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="R188" s="1" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="S188" s="1" t="s">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="T188" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U188" s="1" t="s">
-        <x:v>501</x:v>
-      </x:c>
-      <x:c r="V188" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="W188" s="3">
-        <x:v>46126</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="189" spans="1:29">
@@ -13923,16 +13984,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B189" s="1" t="n">
-        <x:v>36370</x:v>
+        <x:v>36371</x:v>
       </x:c>
       <x:c r="C189" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D189" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E189" s="1" t="s">
-        <x:v>502</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="F189" s="1" t="s">
         <x:v>51</x:v>
@@ -13941,16 +14002,16 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="I189" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J189" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L189" s="4">
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M189" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="190" spans="1:29">
@@ -13958,16 +14019,16 @@
         <x:v>46085.4171919792</x:v>
       </x:c>
       <x:c r="B190" s="1" t="n">
-        <x:v>36371</x:v>
+        <x:v>36372</x:v>
       </x:c>
       <x:c r="C190" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D190" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E190" s="1" t="s">
-        <x:v>503</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="F190" s="1" t="s">
         <x:v>51</x:v>
@@ -13985,30 +14046,33 @@
         <x:v>46085.4124951389</x:v>
       </x:c>
       <x:c r="M190" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="191" spans="1:29">
       <x:c r="A191" s="4">
-        <x:v>46085.4171919792</x:v>
+        <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B191" s="1" t="n">
-        <x:v>36372</x:v>
+        <x:v>36373</x:v>
       </x:c>
       <x:c r="C191" s="1" t="s">
-        <x:v>98</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D191" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E191" s="1" t="s">
-        <x:v>504</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="F191" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="G191" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="H191" s="1" t="s">
+        <x:v>510</x:v>
       </x:c>
       <x:c r="I191" s="1" t="n">
         <x:v>2</x:v>
@@ -14016,11 +14080,44 @@
       <x:c r="J191" s="1" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="K191" s="4">
+        <x:v>46086.7622765857</x:v>
+      </x:c>
       <x:c r="L191" s="4">
-        <x:v>46085.4124951389</x:v>
+        <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M191" s="1" t="s">
-        <x:v>487</x:v>
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="N191" s="4">
+        <x:v>46090.4456414005</x:v>
+      </x:c>
+      <x:c r="O191" s="1" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="P191" s="1" t="n">
+        <x:v>88.87</x:v>
+      </x:c>
+      <x:c r="Q191" s="1" t="n">
+        <x:v>705.36119</x:v>
+      </x:c>
+      <x:c r="R191" s="1" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="S191" s="1" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="T191" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U191" s="1" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="V191" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W191" s="3">
+        <x:v>46095</x:v>
       </x:c>
     </x:row>
     <x:row r="192" spans="1:29">
@@ -14028,25 +14125,25 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B192" s="1" t="n">
-        <x:v>36373</x:v>
+        <x:v>36374</x:v>
       </x:c>
       <x:c r="C192" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
       <x:c r="D192" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E192" s="1" t="s">
-        <x:v>505</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="F192" s="1" t="s">
-        <x:v>506</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="G192" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H192" s="1" t="s">
-        <x:v>507</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="I192" s="1" t="n">
         <x:v>2</x:v>
@@ -14061,7 +14158,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M192" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="N192" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14070,16 +14167,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P192" s="1" t="n">
-        <x:v>88.87</x:v>
+        <x:v>2.51</x:v>
       </x:c>
       <x:c r="Q192" s="1" t="n">
-        <x:v>705.36119</x:v>
+        <x:v>19.92187</x:v>
       </x:c>
       <x:c r="R192" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S192" s="1" t="s">
-        <x:v>509</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="T192" s="1" t="n">
         <x:v>1</x:v>
@@ -14099,25 +14196,25 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B193" s="1" t="n">
-        <x:v>36374</x:v>
+        <x:v>36375</x:v>
       </x:c>
       <x:c r="C193" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
       <x:c r="D193" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E193" s="1" t="s">
-        <x:v>510</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="F193" s="1" t="s">
-        <x:v>511</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="G193" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
       <x:c r="H193" s="1" t="s">
-        <x:v>512</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="I193" s="1" t="n">
         <x:v>2</x:v>
@@ -14132,7 +14229,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M193" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="N193" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14141,16 +14238,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P193" s="1" t="n">
-        <x:v>2.51</x:v>
+        <x:v>5.72</x:v>
       </x:c>
       <x:c r="Q193" s="1" t="n">
-        <x:v>19.92187</x:v>
+        <x:v>45.39964</x:v>
       </x:c>
       <x:c r="R193" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S193" s="1" t="s">
-        <x:v>509</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="T193" s="1" t="n">
         <x:v>1</x:v>
@@ -14170,16 +14267,16 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B194" s="1" t="n">
-        <x:v>36375</x:v>
+        <x:v>36376</x:v>
       </x:c>
       <x:c r="C194" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
       <x:c r="D194" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E194" s="1" t="s">
-        <x:v>513</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="F194" s="1" t="s">
         <x:v>222</x:v>
@@ -14188,7 +14285,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="H194" s="1" t="s">
-        <x:v>514</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="I194" s="1" t="n">
         <x:v>2</x:v>
@@ -14203,7 +14300,7 @@
         <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M194" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="N194" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14212,16 +14309,16 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P194" s="1" t="n">
-        <x:v>5.72</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="Q194" s="1" t="n">
-        <x:v>45.39964</x:v>
+        <x:v>7.1433</x:v>
       </x:c>
       <x:c r="R194" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S194" s="1" t="s">
-        <x:v>509</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="T194" s="1" t="n">
         <x:v>1</x:v>
@@ -14241,40 +14338,28 @@
         <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B195" s="1" t="n">
-        <x:v>36376</x:v>
+        <x:v>36508</x:v>
       </x:c>
       <x:c r="C195" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="D195" s="1" t="s">
-        <x:v>485</x:v>
-      </x:c>
       <x:c r="E195" s="1" t="s">
-        <x:v>515</x:v>
-      </x:c>
-      <x:c r="F195" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="G195" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="H195" s="1" t="s">
-        <x:v>516</x:v>
-      </x:c>
-      <x:c r="I195" s="1" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="J195" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K195" s="4">
-        <x:v>46086.7622765857</x:v>
+        <x:v>46086.6518195255</x:v>
       </x:c>
       <x:c r="L195" s="4">
-        <x:v>46086.7622771991</x:v>
+        <x:v>46086.6518199421</x:v>
       </x:c>
       <x:c r="M195" s="1" t="s">
-        <x:v>508</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="N195" s="4">
         <x:v>46090.4456414005</x:v>
@@ -14283,25 +14368,25 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="P195" s="1" t="n">
-        <x:v>0.9</x:v>
+        <x:v>52.64</x:v>
       </x:c>
       <x:c r="Q195" s="1" t="n">
-        <x:v>7.1433</x:v>
+        <x:v>208.90184</x:v>
       </x:c>
       <x:c r="R195" s="1" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="S195" s="1" t="s">
-        <x:v>509</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="T195" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="U195" s="1" t="s">
         <x:v>228</x:v>
       </x:c>
       <x:c r="V195" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W195" s="3">
         <x:v>46095</x:v>
@@ -14309,155 +14394,131 @@
     </x:row>
     <x:row r="196" spans="1:29">
       <x:c r="A196" s="4">
-        <x:v>46090.4467435532</x:v>
+        <x:v>46087.3857842245</x:v>
       </x:c>
       <x:c r="B196" s="1" t="n">
-        <x:v>36508</x:v>
+        <x:v>36516</x:v>
       </x:c>
       <x:c r="C196" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D196" s="1" t="s">
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E196" s="1" t="s">
-        <x:v>517</x:v>
+        <x:v>521</x:v>
+      </x:c>
+      <x:c r="F196" s="1" t="s">
+        <x:v>64</x:v>
       </x:c>
       <x:c r="G196" s="1" t="s">
-        <x:v>127</x:v>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I196" s="1" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J196" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K196" s="4">
-        <x:v>46086.6518195255</x:v>
-      </x:c>
       <x:c r="L196" s="4">
-        <x:v>46086.6518199421</x:v>
+        <x:v>46086.7566555556</x:v>
       </x:c>
       <x:c r="M196" s="1" t="s">
-        <x:v>418</x:v>
-      </x:c>
-      <x:c r="N196" s="4">
-        <x:v>46090.4456414005</x:v>
-      </x:c>
-      <x:c r="O196" s="1" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="P196" s="1" t="n">
-        <x:v>52.64</x:v>
-      </x:c>
-      <x:c r="Q196" s="1" t="n">
-        <x:v>208.90184</x:v>
-      </x:c>
-      <x:c r="R196" s="1" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="S196" s="1" t="s">
-        <x:v>419</x:v>
-      </x:c>
-      <x:c r="T196" s="1" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="U196" s="1" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="V196" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W196" s="3">
-        <x:v>46095</x:v>
+        <x:v>522</x:v>
       </x:c>
     </x:row>
     <x:row r="197" spans="1:29">
       <x:c r="A197" s="4">
-        <x:v>46087.3857842245</x:v>
+        <x:v>46090.4467435532</x:v>
       </x:c>
       <x:c r="B197" s="1" t="n">
-        <x:v>36516</x:v>
+        <x:v>36518</x:v>
       </x:c>
       <x:c r="C197" s="1" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="D197" s="1" t="s">
-        <x:v>485</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E197" s="1" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="F197" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="G197" s="1" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="I197" s="1" t="n">
-        <x:v>1</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="J197" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="K197" s="4">
+        <x:v>46086.7622765857</x:v>
+      </x:c>
       <x:c r="L197" s="4">
-        <x:v>46086.7566555556</x:v>
+        <x:v>46086.7622771991</x:v>
       </x:c>
       <x:c r="M197" s="1" t="s">
-        <x:v>519</x:v>
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="N197" s="4">
+        <x:v>46090.4456414005</x:v>
+      </x:c>
+      <x:c r="O197" s="1" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="P197" s="1" t="n">
+        <x:v>92.08</x:v>
+      </x:c>
+      <x:c r="Q197" s="1" t="n">
+        <x:v>365.41948</x:v>
+      </x:c>
+      <x:c r="R197" s="1" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="S197" s="1" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="T197" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U197" s="1" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="V197" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W197" s="3">
+        <x:v>46095</x:v>
       </x:c>
     </x:row>
     <x:row r="198" spans="1:29">
       <x:c r="A198" s="4">
-        <x:v>46090.4467435532</x:v>
+        <x:v>46100.4842279745</x:v>
       </x:c>
       <x:c r="B198" s="1" t="n">
-        <x:v>36518</x:v>
+        <x:v>37261</x:v>
       </x:c>
       <x:c r="C198" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="D198" s="1" t="s">
+        <x:v>524</x:v>
       </x:c>
       <x:c r="E198" s="1" t="s">
-        <x:v>520</x:v>
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="F198" s="1" t="s">
+        <x:v>64</x:v>
       </x:c>
       <x:c r="G198" s="1" t="s">
-        <x:v>127</x:v>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I198" s="1" t="n">
+        <x:v>9</x:v>
       </x:c>
       <x:c r="J198" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K198" s="4">
-        <x:v>46086.7622765857</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="L198" s="4">
-        <x:v>46086.7622771991</x:v>
+        <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M198" s="1" t="s">
-        <x:v>508</x:v>
-      </x:c>
-      <x:c r="N198" s="4">
-        <x:v>46090.4456414005</x:v>
-      </x:c>
-      <x:c r="O198" s="1" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="P198" s="1" t="n">
-        <x:v>92.08</x:v>
-      </x:c>
-      <x:c r="Q198" s="1" t="n">
-        <x:v>365.41948</x:v>
-      </x:c>
-      <x:c r="R198" s="1" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="S198" s="1" t="s">
-        <x:v>509</x:v>
-      </x:c>
-      <x:c r="T198" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U198" s="1" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="V198" s="1" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W198" s="3">
-        <x:v>46095</x:v>
+        <x:v>526</x:v>
       </x:c>
     </x:row>
     <x:row r="199" spans="1:29">
@@ -14465,16 +14526,16 @@
         <x:v>46100.4842279745</x:v>
       </x:c>
       <x:c r="B199" s="1" t="n">
-        <x:v>37261</x:v>
+        <x:v>37262</x:v>
       </x:c>
       <x:c r="C199" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D199" s="1" t="s">
-        <x:v>521</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="E199" s="1" t="s">
-        <x:v>522</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="F199" s="1" t="s">
         <x:v>64</x:v>
@@ -14483,16 +14544,16 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="I199" s="1" t="n">
-        <x:v>9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J199" s="1" t="n">
-        <x:v>9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L199" s="4">
         <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M199" s="1" t="s">
-        <x:v>523</x:v>
+        <x:v>526</x:v>
       </x:c>
     </x:row>
     <x:row r="200" spans="1:29">
@@ -14500,16 +14561,16 @@
         <x:v>46100.4842279745</x:v>
       </x:c>
       <x:c r="B200" s="1" t="n">
-        <x:v>37262</x:v>
+        <x:v>37265</x:v>
       </x:c>
       <x:c r="C200" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D200" s="1" t="s">
-        <x:v>521</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="E200" s="1" t="s">
-        <x:v>524</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="F200" s="1" t="s">
         <x:v>64</x:v>
@@ -14518,16 +14579,16 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="I200" s="1" t="n">
-        <x:v>18</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J200" s="1" t="n">
-        <x:v>18</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L200" s="4">
         <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M200" s="1" t="s">
-        <x:v>523</x:v>
+        <x:v>526</x:v>
       </x:c>
     </x:row>
     <x:row r="201" spans="1:29">
@@ -14535,16 +14596,16 @@
         <x:v>46100.4842279745</x:v>
       </x:c>
       <x:c r="B201" s="1" t="n">
-        <x:v>37265</x:v>
+        <x:v>37266</x:v>
       </x:c>
       <x:c r="C201" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D201" s="1" t="s">
-        <x:v>521</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="E201" s="1" t="s">
-        <x:v>525</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F201" s="1" t="s">
         <x:v>64</x:v>
@@ -14562,42 +14623,42 @@
         <x:v>46098.5238698727</x:v>
       </x:c>
       <x:c r="M201" s="1" t="s">
-        <x:v>523</x:v>
+        <x:v>526</x:v>
       </x:c>
     </x:row>
     <x:row r="202" spans="1:29">
       <x:c r="A202" s="4">
-        <x:v>46100.4842279745</x:v>
+        <x:v>46100.4847336806</x:v>
       </x:c>
       <x:c r="B202" s="1" t="n">
-        <x:v>37266</x:v>
+        <x:v>37412</x:v>
       </x:c>
       <x:c r="C202" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D202" s="1" t="s">
-        <x:v>521</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="E202" s="1" t="s">
-        <x:v>526</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="F202" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G202" s="1" t="s">
         <x:v>52</x:v>
       </x:c>
       <x:c r="I202" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J202" s="1" t="n">
-        <x:v>2</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L202" s="4">
-        <x:v>46098.5238698727</x:v>
+        <x:v>46100.4729106481</x:v>
       </x:c>
       <x:c r="M202" s="1" t="s">
-        <x:v>523</x:v>
+        <x:v>531</x:v>
       </x:c>
     </x:row>
     <x:row r="203" spans="1:29">
@@ -14605,16 +14666,16 @@
         <x:v>46100.4847336806</x:v>
       </x:c>
       <x:c r="B203" s="1" t="n">
-        <x:v>37412</x:v>
+        <x:v>37413</x:v>
       </x:c>
       <x:c r="C203" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
       <x:c r="D203" s="1" t="s">
-        <x:v>521</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="E203" s="1" t="s">
-        <x:v>527</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="F203" s="1" t="s">
         <x:v>51</x:v>
@@ -14623,51 +14684,16 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="I203" s="1" t="n">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J203" s="1" t="n">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="L203" s="4">
         <x:v>46100.4729106481</x:v>
       </x:c>
       <x:c r="M203" s="1" t="s">
-        <x:v>528</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="204" spans="1:29">
-      <x:c r="A204" s="4">
-        <x:v>46100.4847336806</x:v>
-      </x:c>
-      <x:c r="B204" s="1" t="n">
-        <x:v>37413</x:v>
-      </x:c>
-      <x:c r="C204" s="1" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="D204" s="1" t="s">
-        <x:v>521</x:v>
-      </x:c>
-      <x:c r="E204" s="1" t="s">
-        <x:v>529</x:v>
-      </x:c>
-      <x:c r="F204" s="1" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G204" s="1" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="I204" s="1" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="J204" s="1" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="L204" s="4">
-        <x:v>46100.4729106481</x:v>
-      </x:c>
-      <x:c r="M204" s="1" t="s">
-        <x:v>528</x:v>
+        <x:v>531</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>